<commit_message>
Load 2026 Harrison Landing ad spend actuals
Digible $2,295/mo and Zillow $958/mo become 2027 fixed fees; CoStar is
cancelled (last invoice 9/30/26) with its lease share moved to Zillow.
Adds 2026 actuals by channel and a comparison to the 2026 ad budget.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S4EZy9r3vcic7sA8Y6yuUD
</commit_message>
<xml_diff>
--- a/Harrison_Landing_2027_Marketing_Budget.xlsx
+++ b/Harrison_Landing_2027_Marketing_Budget.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -585,86 +585,94 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Budget per unit per year</t>
+          <t>2027 paid lead-channel spend</t>
         </is>
       </c>
       <c r="B6" s="9">
-        <f>IFERROR(B5/Inputs!$B$9,0)</f>
-        <v/>
-      </c>
-      <c r="E6" s="7" t="inlineStr"/>
+        <f>'Monthly Plan'!$N$37</f>
+        <v/>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Compare: 2026 actual $53,958, 2026 budget $43,758</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Budget per unit per month</t>
-        </is>
-      </c>
-      <c r="B7" s="10">
-        <f>IFERROR(B5/Inputs!$B$9/12,0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="7" t="inlineStr"/>
+          <t>vs. 2026 budgeted ad spend</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>B6-Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Positive = more than the 2026 budget</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
+          <t>Budget per unit per year</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>IFERROR(B5/Inputs!$B$9,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Budget per unit per month</t>
+        </is>
+      </c>
+      <c r="B9" s="10">
+        <f>IFERROR(B5/Inputs!$B$9/12,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
           <t>% of gross potential rent</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B10" s="11">
         <f>IFERROR(B5/(Inputs!$B$9*Inputs!$B$10*12),0)</f>
         <v/>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Many operators land ~1–3% of GPR</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Lease demand</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Leases expiring in 2027</t>
-        </is>
-      </c>
-      <c r="B11" s="12">
-        <f>'Monthly Plan'!$N$7</f>
-        <v/>
-      </c>
-      <c r="E11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Renewals</t>
-        </is>
-      </c>
-      <c r="B12" s="12">
-        <f>'Monthly Plan'!$N$8</f>
-        <v/>
-      </c>
-      <c r="E12" s="7" t="inlineStr"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Move-outs (expirations + early terminations)</t>
+          <t>Leases expiring in 2027</t>
         </is>
       </c>
       <c r="B13" s="12">
-        <f>'Monthly Plan'!$N$9+'Monthly Plan'!$N$10</f>
+        <f>'Monthly Plan'!$N$7</f>
         <v/>
       </c>
       <c r="E13" s="7" t="inlineStr"/>
@@ -672,27 +680,23 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Implied annual turnover rate</t>
-        </is>
-      </c>
-      <c r="B14" s="11">
-        <f>IFERROR(B13/Inputs!$B$9,0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Move-outs ÷ total units</t>
-        </is>
-      </c>
+          <t>Renewals</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>'Monthly Plan'!$N$8</f>
+        <v/>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>New leases needed</t>
-        </is>
-      </c>
-      <c r="B15" s="13">
-        <f>'Monthly Plan'!$N$12</f>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Move-outs (expirations + early terminations)</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>'Monthly Plan'!$N$9+'Monthly Plan'!$N$10</f>
         <v/>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
@@ -700,27 +704,27 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Blended lead-to-lease rate (channel mix)</t>
+          <t>Implied annual turnover rate</t>
         </is>
       </c>
       <c r="B16" s="11">
-        <f>IFERROR(B15/'Monthly Plan'!$N$23,0)</f>
+        <f>IFERROR(B15/Inputs!$B$9,0)</f>
         <v/>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>New leases ÷ leads</t>
+          <t>Move-outs ÷ total units</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Leads needed</t>
+          <t>New leases needed</t>
         </is>
       </c>
       <c r="B17" s="13">
-        <f>'Monthly Plan'!$N$23</f>
+        <f>'Monthly Plan'!$N$12</f>
         <v/>
       </c>
       <c r="E17" s="7" t="inlineStr"/>
@@ -728,321 +732,281 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>Blended lead-to-lease rate (channel mix)</t>
+        </is>
+      </c>
+      <c r="B18" s="11">
+        <f>IFERROR(B17/'Monthly Plan'!$N$23,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>New leases ÷ leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Leads needed</t>
+        </is>
+      </c>
+      <c r="B19" s="13">
+        <f>'Monthly Plan'!$N$23</f>
+        <v/>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
           <t>Tours needed</t>
         </is>
       </c>
-      <c r="B18" s="12">
+      <c r="B20" s="12">
         <f>'Monthly Plan'!$N$25</f>
         <v/>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Efficiency checks</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Blended cost per lead</t>
-        </is>
-      </c>
-      <c r="B21" s="10">
-        <f>IFERROR('Monthly Plan'!$N$37/B17,0)</f>
-        <v/>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Channel spend ÷ leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Cost per new lease (all-in)</t>
-        </is>
-      </c>
-      <c r="B22" s="14">
-        <f>IFERROR(B5/B15,0)</f>
-        <v/>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Total budget ÷ new leases</t>
-        </is>
-      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Cost per lease as % of one month's rent</t>
-        </is>
-      </c>
-      <c r="B23" s="11">
-        <f>IFERROR(B22/Inputs!$B$10,0)</f>
-        <v/>
-      </c>
-      <c r="E23" s="7" t="inlineStr"/>
+          <t>Blended cost per lead</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>IFERROR('Monthly Plan'!$N$37/B19,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Channel spend ÷ leads</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Within cost-per-lease target?</t>
-        </is>
-      </c>
-      <c r="B24" s="15">
-        <f>IF(B23&lt;=Inputs!$B$34,"YES","OVER TARGET")</f>
-        <v/>
-      </c>
-      <c r="E24" s="7" t="inlineStr"/>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Cost per new lease (all-in)</t>
+        </is>
+      </c>
+      <c r="B24" s="14">
+        <f>IFERROR(B5/B17,0)</f>
+        <v/>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Total budget ÷ new leases</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
+          <t>Cost per lease as % of one month's rent</t>
+        </is>
+      </c>
+      <c r="B25" s="11">
+        <f>IFERROR(B24/Inputs!$B$10,0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Within cost-per-lease target?</t>
+        </is>
+      </c>
+      <c r="B26" s="15">
+        <f>IF(B25&lt;=Inputs!$B$35,"YES","OVER TARGET")</f>
+        <v/>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
           <t>Stress test: leads needed at T-3 conversion</t>
         </is>
       </c>
-      <c r="B25" s="12">
-        <f>IFERROR(B15/Inputs!$B$27,0)</f>
-        <v/>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="B27" s="12">
+        <f>IFERROR(B17/Inputs!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>If the recent 1.3% conversion continues</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Stress test: extra per-lead spend at T-3 conversion</t>
         </is>
       </c>
-      <c r="B26" s="14">
-        <f>MAX(0,(B25-B17)*B21)</f>
-        <v/>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="B28" s="14">
+        <f>MAX(0,(B27-B19)*B23)</f>
+        <v/>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>Extra leads × blended cost per lead. Fixing conversion is cheaper</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Why it pays: cost of vacancy</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Projected 2027 vacancy loss from turns</t>
-        </is>
-      </c>
-      <c r="B29" s="9">
-        <f>B13*Inputs!$B$13*Inputs!$B$10/30</f>
-        <v/>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Move-outs × days vacant × daily rent</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Value of cutting 1 vacant day per turn</t>
-        </is>
-      </c>
-      <c r="B30" s="9">
-        <f>B13*Inputs!$B$10/30</f>
-        <v/>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Use this to justify spend that speeds up leasing</t>
-        </is>
-      </c>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Concession cost on new leases (memo)</t>
+          <t>Projected 2027 vacancy loss from turns</t>
         </is>
       </c>
       <c r="B31" s="9">
-        <f>B15*Inputs!$B$30*Inputs!$B$10*12/52</f>
+        <f>B15*Inputs!$B$13*Inputs!$B$10/30</f>
         <v/>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Not in marketing budget. Weeks free × weekly rent × new leases</t>
+          <t>Move-outs × days vacant × daily rent</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
+          <t>Value of cutting 1 vacant day per turn</t>
+        </is>
+      </c>
+      <c r="B32" s="9">
+        <f>B15*Inputs!$B$10/30</f>
+        <v/>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Use this to justify spend that speeds up leasing</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Concession cost on new leases (memo)</t>
+        </is>
+      </c>
+      <c r="B33" s="9">
+        <f>B17*Inputs!$B$31*Inputs!$B$10*12/52</f>
+        <v/>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Not in marketing budget. Weeks free × weekly rent × new leases</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>Value of +5 pts renewal rate</t>
         </is>
       </c>
-      <c r="B32" s="9">
-        <f>B11*0.05*(Inputs!$B$13*Inputs!$B$10/30+IFERROR(B22,0))</f>
-        <v/>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="B34" s="9">
+        <f>B13*0.05*(Inputs!$B$13*Inputs!$B$10/30+IFERROR(B24,0))</f>
+        <v/>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>Avoided vacancy + avoided acquisition cost</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Budget by line item</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Line item</t>
         </is>
       </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>2027 Budget ($)</t>
         </is>
       </c>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>2026 Actual ($)</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Variance ($)</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Share of budget</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>2027 leads</t>
         </is>
       </c>
-      <c r="G35" s="16" t="inlineStr">
+      <c r="G37" s="16" t="inlineStr">
         <is>
           <t>2027 leases</t>
         </is>
       </c>
-      <c r="H35" s="16" t="inlineStr">
+      <c r="H37" s="16" t="inlineStr">
         <is>
           <t>Cost per lease ($)</t>
         </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17">
-        <f>Inputs!$A$54</f>
-        <v/>
-      </c>
-      <c r="B36" s="9">
-        <f>'Monthly Plan'!$N$28</f>
-        <v/>
-      </c>
-      <c r="C36" s="9">
-        <f>IF(Inputs!$G$54="","",Inputs!$G$54)</f>
-        <v/>
-      </c>
-      <c r="D36" s="18">
-        <f>IF(C36="","",B36-C36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="19">
-        <f>IFERROR(B36/B5,0)</f>
-        <v/>
-      </c>
-      <c r="F36" s="12">
-        <f>'Monthly Plan'!$N$14</f>
-        <v/>
-      </c>
-      <c r="G36" s="20">
-        <f>B15*Inputs!$B$54</f>
-        <v/>
-      </c>
-      <c r="H36" s="18">
-        <f>IFERROR(B36/G36,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="17">
-        <f>Inputs!$A$55</f>
-        <v/>
-      </c>
-      <c r="B37" s="9">
-        <f>'Monthly Plan'!$N$29</f>
-        <v/>
-      </c>
-      <c r="C37" s="9">
-        <f>IF(Inputs!$G$55="","",Inputs!$G$55)</f>
-        <v/>
-      </c>
-      <c r="D37" s="18">
-        <f>IF(C37="","",B37-C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="19">
-        <f>IFERROR(B37/B5,0)</f>
-        <v/>
-      </c>
-      <c r="F37" s="12">
-        <f>'Monthly Plan'!$N$15</f>
-        <v/>
-      </c>
-      <c r="G37" s="20">
-        <f>B15*Inputs!$B$55</f>
-        <v/>
-      </c>
-      <c r="H37" s="18">
-        <f>IFERROR(B37/G37,0)</f>
-        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="17">
-        <f>Inputs!$A$56</f>
+        <f>Inputs!$A$55</f>
         <v/>
       </c>
       <c r="B38" s="9">
-        <f>'Monthly Plan'!$N$30</f>
+        <f>'Monthly Plan'!$N$28</f>
         <v/>
       </c>
       <c r="C38" s="9">
-        <f>IF(Inputs!$G$56="","",Inputs!$G$56)</f>
+        <f>IF(Inputs!$G$55="","",Inputs!$G$55)</f>
         <v/>
       </c>
       <c r="D38" s="18">
@@ -1054,11 +1018,11 @@
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>'Monthly Plan'!$N$16</f>
+        <f>'Monthly Plan'!$N$14</f>
         <v/>
       </c>
       <c r="G38" s="20">
-        <f>B15*Inputs!$B$56</f>
+        <f>B17*Inputs!$B$55</f>
         <v/>
       </c>
       <c r="H38" s="18">
@@ -1068,15 +1032,15 @@
     </row>
     <row r="39">
       <c r="A39" s="17">
-        <f>Inputs!$A$57</f>
+        <f>Inputs!$A$56</f>
         <v/>
       </c>
       <c r="B39" s="9">
-        <f>'Monthly Plan'!$N$31</f>
+        <f>'Monthly Plan'!$N$29</f>
         <v/>
       </c>
       <c r="C39" s="9">
-        <f>IF(Inputs!$G$57="","",Inputs!$G$57)</f>
+        <f>IF(Inputs!$G$56="","",Inputs!$G$56)</f>
         <v/>
       </c>
       <c r="D39" s="18">
@@ -1088,11 +1052,11 @@
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>'Monthly Plan'!$N$17</f>
+        <f>'Monthly Plan'!$N$15</f>
         <v/>
       </c>
       <c r="G39" s="20">
-        <f>B15*Inputs!$B$57</f>
+        <f>B17*Inputs!$B$56</f>
         <v/>
       </c>
       <c r="H39" s="18">
@@ -1102,15 +1066,15 @@
     </row>
     <row r="40">
       <c r="A40" s="17">
-        <f>Inputs!$A$58</f>
+        <f>Inputs!$A$57</f>
         <v/>
       </c>
       <c r="B40" s="9">
-        <f>'Monthly Plan'!$N$32</f>
+        <f>'Monthly Plan'!$N$30</f>
         <v/>
       </c>
       <c r="C40" s="9">
-        <f>IF(Inputs!$G$58="","",Inputs!$G$58)</f>
+        <f>IF(Inputs!$G$57="","",Inputs!$G$57)</f>
         <v/>
       </c>
       <c r="D40" s="18">
@@ -1122,11 +1086,11 @@
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>'Monthly Plan'!$N$18</f>
+        <f>'Monthly Plan'!$N$16</f>
         <v/>
       </c>
       <c r="G40" s="20">
-        <f>B15*Inputs!$B$58</f>
+        <f>B17*Inputs!$B$57</f>
         <v/>
       </c>
       <c r="H40" s="18">
@@ -1136,15 +1100,15 @@
     </row>
     <row r="41">
       <c r="A41" s="17">
-        <f>Inputs!$A$59</f>
+        <f>Inputs!$A$58</f>
         <v/>
       </c>
       <c r="B41" s="9">
-        <f>'Monthly Plan'!$N$33</f>
+        <f>'Monthly Plan'!$N$31</f>
         <v/>
       </c>
       <c r="C41" s="9">
-        <f>IF(Inputs!$G$59="","",Inputs!$G$59)</f>
+        <f>IF(Inputs!$G$58="","",Inputs!$G$58)</f>
         <v/>
       </c>
       <c r="D41" s="18">
@@ -1156,11 +1120,11 @@
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>'Monthly Plan'!$N$19</f>
+        <f>'Monthly Plan'!$N$17</f>
         <v/>
       </c>
       <c r="G41" s="20">
-        <f>B15*Inputs!$B$59</f>
+        <f>B17*Inputs!$B$58</f>
         <v/>
       </c>
       <c r="H41" s="18">
@@ -1170,15 +1134,15 @@
     </row>
     <row r="42">
       <c r="A42" s="17">
-        <f>Inputs!$A$60</f>
+        <f>Inputs!$A$59</f>
         <v/>
       </c>
       <c r="B42" s="9">
-        <f>'Monthly Plan'!$N$34</f>
+        <f>'Monthly Plan'!$N$32</f>
         <v/>
       </c>
       <c r="C42" s="9">
-        <f>IF(Inputs!$G$60="","",Inputs!$G$60)</f>
+        <f>IF(Inputs!$G$59="","",Inputs!$G$59)</f>
         <v/>
       </c>
       <c r="D42" s="18">
@@ -1190,11 +1154,11 @@
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>'Monthly Plan'!$N$20</f>
+        <f>'Monthly Plan'!$N$18</f>
         <v/>
       </c>
       <c r="G42" s="20">
-        <f>B15*Inputs!$B$60</f>
+        <f>B17*Inputs!$B$59</f>
         <v/>
       </c>
       <c r="H42" s="18">
@@ -1204,15 +1168,15 @@
     </row>
     <row r="43">
       <c r="A43" s="17">
-        <f>Inputs!$A$61</f>
+        <f>Inputs!$A$60</f>
         <v/>
       </c>
       <c r="B43" s="9">
-        <f>'Monthly Plan'!$N$35</f>
+        <f>'Monthly Plan'!$N$33</f>
         <v/>
       </c>
       <c r="C43" s="9">
-        <f>IF(Inputs!$G$61="","",Inputs!$G$61)</f>
+        <f>IF(Inputs!$G$60="","",Inputs!$G$60)</f>
         <v/>
       </c>
       <c r="D43" s="18">
@@ -1224,11 +1188,11 @@
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>'Monthly Plan'!$N$21</f>
+        <f>'Monthly Plan'!$N$19</f>
         <v/>
       </c>
       <c r="G43" s="20">
-        <f>B15*Inputs!$B$61</f>
+        <f>B17*Inputs!$B$60</f>
         <v/>
       </c>
       <c r="H43" s="18">
@@ -1238,15 +1202,15 @@
     </row>
     <row r="44">
       <c r="A44" s="17">
-        <f>Inputs!$A$62</f>
+        <f>Inputs!$A$61</f>
         <v/>
       </c>
       <c r="B44" s="9">
-        <f>'Monthly Plan'!$N$36</f>
+        <f>'Monthly Plan'!$N$34</f>
         <v/>
       </c>
       <c r="C44" s="9">
-        <f>IF(Inputs!$G$62="","",Inputs!$G$62)</f>
+        <f>IF(Inputs!$G$61="","",Inputs!$G$61)</f>
         <v/>
       </c>
       <c r="D44" s="18">
@@ -1258,11 +1222,11 @@
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>'Monthly Plan'!$N$22</f>
+        <f>'Monthly Plan'!$N$20</f>
         <v/>
       </c>
       <c r="G44" s="20">
-        <f>B15*Inputs!$B$62</f>
+        <f>B17*Inputs!$B$61</f>
         <v/>
       </c>
       <c r="H44" s="18">
@@ -1271,85 +1235,153 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>Fixed, program &amp; retention costs</t>
-        </is>
+      <c r="A45" s="17">
+        <f>Inputs!$A$62</f>
+        <v/>
       </c>
       <c r="B45" s="9">
-        <f>'Monthly Plan'!$N$49</f>
+        <f>'Monthly Plan'!$N$35</f>
+        <v/>
+      </c>
+      <c r="C45" s="9">
+        <f>IF(Inputs!$G$62="","",Inputs!$G$62)</f>
+        <v/>
+      </c>
+      <c r="D45" s="18">
+        <f>IF(C45="","",B45-C45)</f>
         <v/>
       </c>
       <c r="E45" s="19">
         <f>IFERROR(B45/B5,0)</f>
         <v/>
       </c>
+      <c r="F45" s="12">
+        <f>'Monthly Plan'!$N$21</f>
+        <v/>
+      </c>
+      <c r="G45" s="20">
+        <f>B17*Inputs!$B$62</f>
+        <v/>
+      </c>
+      <c r="H45" s="18">
+        <f>IFERROR(B45/G45,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
+      <c r="A46" s="17">
+        <f>Inputs!$A$63</f>
+        <v/>
       </c>
       <c r="B46" s="9">
-        <f>'Monthly Plan'!$N$52</f>
+        <f>'Monthly Plan'!$N$36</f>
+        <v/>
+      </c>
+      <c r="C46" s="9">
+        <f>IF(Inputs!$G$63="","",Inputs!$G$63)</f>
+        <v/>
+      </c>
+      <c r="D46" s="18">
+        <f>IF(C46="","",B46-C46)</f>
         <v/>
       </c>
       <c r="E46" s="19">
         <f>IFERROR(B46/B5,0)</f>
         <v/>
       </c>
+      <c r="F46" s="12">
+        <f>'Monthly Plan'!$N$22</f>
+        <v/>
+      </c>
+      <c r="G46" s="20">
+        <f>B17*Inputs!$B$63</f>
+        <v/>
+      </c>
+      <c r="H46" s="18">
+        <f>IFERROR(B46/G46,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="21" t="inlineStr">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Fixed, program &amp; retention costs</t>
+        </is>
+      </c>
+      <c r="B47" s="9">
+        <f>'Monthly Plan'!$N$49</f>
+        <v/>
+      </c>
+      <c r="E47" s="19">
+        <f>IFERROR(B47/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B48" s="9">
+        <f>'Monthly Plan'!$N$52</f>
+        <v/>
+      </c>
+      <c r="E48" s="19">
+        <f>IFERROR(B48/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B47" s="22">
-        <f>SUM(B36:B46)</f>
-        <v/>
-      </c>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="23" t="n"/>
-      <c r="E47" s="24">
-        <f>SUM(E36:E46)</f>
-        <v/>
-      </c>
-      <c r="F47" s="23" t="n"/>
-      <c r="G47" s="23" t="n"/>
-      <c r="H47" s="23" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="B49" s="22">
+        <f>SUM(B38:B48)</f>
+        <v/>
+      </c>
+      <c r="C49" s="23" t="n"/>
+      <c r="D49" s="23" t="n"/>
+      <c r="E49" s="24">
+        <f>SUM(E38:E48)</f>
+        <v/>
+      </c>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="23" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Input checks</t>
         </is>
       </c>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Seasonality sums to 100%</t>
         </is>
       </c>
-      <c r="B50" s="17">
-        <f>Inputs!$C$50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="B52" s="17">
+        <f>Inputs!$C$51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>Channel lease mix sums to 100%</t>
         </is>
       </c>
-      <c r="B51" s="17">
-        <f>Inputs!$C$63</f>
+      <c r="B53" s="17">
+        <f>Inputs!$C$64</f>
         <v/>
       </c>
     </row>
@@ -1364,7 +1396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1808,179 +1840,189 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
+          <t>2026 budgeted ad spend (memo)</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="n">
+        <v>43758</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>ACTUAL: 2026 Ad Spend Tracking. Actual was $53,958; $10,200 over because CoStar billed Apr–Sep after it was cut from budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
           <t>Weeks free offered per new lease</t>
         </is>
       </c>
-      <c r="B30" s="27" t="n">
+      <c r="B31" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>weeks</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>ACTUAL: WAR 10/4/26 current special is 6 weeks free + waived L&amp;L admin</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Budget guardrails</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Contingency / reserve</t>
-        </is>
-      </c>
-      <c r="B33" s="29" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>Cushion for slow months, price hikes, surprise vacancies</t>
-        </is>
-      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
+          <t>Contingency / reserve</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Cushion for slow months, price hikes, surprise vacancies</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>Target max cost per lease (% of one month's rent)</t>
         </is>
       </c>
-      <c r="B34" s="29" t="n">
+      <c r="B35" s="29" t="n">
         <v>0.5</v>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>Common rule of thumb: keep acquisition cost under ~½ month's rent</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Lease expiration seasonality (% of 2027 expirations by month)</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>% of expirations</t>
         </is>
       </c>
-      <c r="C37" s="16" t="inlineStr"/>
-      <c r="D37" s="16" t="inlineStr"/>
-      <c r="E37" s="16" t="inlineStr"/>
-      <c r="F37" s="16" t="inlineStr"/>
-      <c r="G37" s="16" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr"/>
+      <c r="D38" s="16" t="inlineStr"/>
+      <c r="E38" s="16" t="inlineStr"/>
+      <c r="F38" s="16" t="inlineStr"/>
+      <c r="G38" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B38" s="29" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER curve (summer-heavy). Replace with actual 2027 expiration counts by month.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B39" s="29" t="n">
         <v>0.05</v>
       </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER curve (summer-heavy). Replace with actual 2027 expiration counts by month.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="B40" s="29" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="B41" s="29" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B42" s="29" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B43" s="29" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="B44" s="29" t="n">
@@ -1990,215 +2032,193 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B45" s="29" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="B46" s="29" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="B47" s="29" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="B48" s="29" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B49" s="29" t="n">
+      <c r="B50" s="29" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Total (must = 100%)</t>
         </is>
       </c>
-      <c r="B50" s="30">
-        <f>SUM(B38:B49)</f>
-        <v/>
-      </c>
-      <c r="C50" s="5">
-        <f>IF(ROUND(B50,4)=1,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="B51" s="30">
+        <f>SUM(B39:B50)</f>
+        <v/>
+      </c>
+      <c r="C51" s="5">
+        <f>IF(ROUND(B51,4)=1,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Lead channels (2027 lease mix and channel conversion)</t>
         </is>
       </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="B53" s="16" t="inlineStr">
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>% of 2027 new leases</t>
         </is>
       </c>
-      <c r="C53" s="16" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>Channel lead-to-lease</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>Cost per lead ($)</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr">
+      <c r="E54" s="16" t="inlineStr">
         <is>
           <t>Fixed monthly fee ($)</t>
         </is>
       </c>
-      <c r="F53" s="16" t="inlineStr">
+      <c r="F54" s="16" t="inlineStr">
         <is>
           <t>Cost per signed lease ($)</t>
         </is>
       </c>
-      <c r="G53" s="16" t="inlineStr">
+      <c r="G54" s="16" t="inlineStr">
         <is>
           <t>2026 actual spend ($)</t>
         </is>
       </c>
-      <c r="H53" s="16" t="inlineStr">
+      <c r="H54" s="16" t="inlineStr">
         <is>
           <t>T-12 leads (memo)</t>
         </is>
       </c>
-      <c r="I53" s="16" t="inlineStr">
+      <c r="I54" s="16" t="inlineStr">
         <is>
           <t>T-12 leases (memo)</t>
         </is>
       </c>
-      <c r="J53" s="16" t="inlineStr">
+      <c r="J54" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>Zillow</t>
-        </is>
-      </c>
-      <c r="B54" s="29" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C54" s="29" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="D54" s="28" t="n">
-        <v>25</v>
-      </c>
-      <c r="E54" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="28" t="n"/>
-      <c r="H54" s="31" t="n">
-        <v>634</v>
-      </c>
-      <c r="I54" s="31" t="n">
-        <v>14</v>
-      </c>
-      <c r="J54" s="7" t="inlineStr">
-        <is>
-          <t>Mix &amp; conversion ACTUAL (WAR T-12). Cost PLACEHOLDER: confirm Zillow pricing</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Property website</t>
+          <t>Zillow</t>
         </is>
       </c>
       <c r="B55" s="29" t="n">
-        <v>0.232</v>
+        <v>0.268</v>
       </c>
       <c r="C55" s="29" t="n">
-        <v>0.057</v>
+        <v>0.022</v>
       </c>
       <c r="D55" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="28" t="n">
-        <v>0</v>
+        <v>958</v>
       </c>
       <c r="F55" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G55" s="28" t="n"/>
+      <c r="G55" s="28" t="n">
+        <v>11244</v>
+      </c>
       <c r="H55" s="31" t="n">
-        <v>228</v>
+        <v>634</v>
       </c>
       <c r="I55" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Site cost is in fixed costs</t>
+          <t>Mix/conv ACTUAL (WAR T-12). Fee ACTUAL: $958/mo since Oct 2026 (was $930). Mix includes Apts.com's former share</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Property website</t>
         </is>
       </c>
       <c r="B56" s="29" t="n">
-        <v>0.161</v>
+        <v>0.232</v>
       </c>
       <c r="C56" s="29" t="n">
-        <v>0.049</v>
+        <v>0.057</v>
       </c>
       <c r="D56" s="28" t="n">
         <v>0</v>
@@ -2209,30 +2229,32 @@
       <c r="F56" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G56" s="28" t="n"/>
+      <c r="G56" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="H56" s="31" t="n">
-        <v>183</v>
+        <v>228</v>
       </c>
       <c r="I56" s="31" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Cost PLACEHOLDER: any MLS / agent fees?</t>
+          <t>ACTUAL. $0 on ad tracker; hosting is in fixed costs. Digible ads may land here</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>Google (organic / Business Profile)</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="B57" s="29" t="n">
-        <v>0.107</v>
+        <v>0.161</v>
       </c>
       <c r="C57" s="29" t="n">
-        <v>0.128</v>
+        <v>0.049</v>
       </c>
       <c r="D57" s="28" t="n">
         <v>0</v>
@@ -2245,65 +2267,65 @@
       </c>
       <c r="G57" s="28" t="n"/>
       <c r="H57" s="31" t="n">
-        <v>47</v>
+        <v>183</v>
       </c>
       <c r="I57" s="31" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Best converting source</t>
+          <t>ACTUAL mix/conv. Not on ad tracker: any MLS / agent fees?</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>Rently (self-tour listings)</t>
+          <t>Google (organic / Business Profile)</t>
         </is>
       </c>
       <c r="B58" s="29" t="n">
         <v>0.107</v>
       </c>
       <c r="C58" s="29" t="n">
-        <v>0.033</v>
+        <v>0.128</v>
       </c>
       <c r="D58" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="28" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F58" s="28" t="n">
         <v>0</v>
       </c>
       <c r="G58" s="28" t="n"/>
       <c r="H58" s="31" t="n">
-        <v>184</v>
+        <v>47</v>
       </c>
       <c r="I58" s="31" t="n">
         <v>6</v>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Fee PLACEHOLDER</t>
+          <t>ACTUAL mix/conv. Best converting source, $0 cost</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>PPC (paid search)</t>
+          <t>Rently (self-tour listings)</t>
         </is>
       </c>
       <c r="B59" s="29" t="n">
-        <v>0.054</v>
+        <v>0.107</v>
       </c>
       <c r="C59" s="29" t="n">
-        <v>0.029</v>
+        <v>0.033</v>
       </c>
       <c r="D59" s="28" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E59" s="28" t="n">
         <v>0</v>
@@ -2313,62 +2335,64 @@
       </c>
       <c r="G59" s="28" t="n"/>
       <c r="H59" s="31" t="n">
-        <v>103</v>
+        <v>184</v>
       </c>
       <c r="I59" s="31" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. CPL PLACEHOLDER</t>
+          <t>ACTUAL mix/conv. Not on ad tracker: confirm if billed elsewhere</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>Apartments.com / CoStar</t>
+          <t>Digible (PPC / paid digital)</t>
         </is>
       </c>
       <c r="B60" s="29" t="n">
-        <v>0.018</v>
+        <v>0.054</v>
       </c>
       <c r="C60" s="29" t="n">
-        <v>0.008</v>
+        <v>0.029</v>
       </c>
       <c r="D60" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="28" t="n">
-        <v>1200</v>
+        <v>2295</v>
       </c>
       <c r="F60" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G60" s="28" t="n"/>
+      <c r="G60" s="28" t="n">
+        <v>27540</v>
+      </c>
       <c r="H60" s="31" t="n">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="I60" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv: 1 lease from 120 leads. Fee PLACEHOLDER: review before renewing</t>
+          <t>Fee ACTUAL: $2,295/mo. WAR credits PPC with only 3 leases; get Digible's attribution report</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>Apartment List</t>
+          <t>Apartments.com / CoStar</t>
         </is>
       </c>
       <c r="B61" s="29" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="C61" s="29" t="n">
-        <v>0.083</v>
+        <v>0.008</v>
       </c>
       <c r="D61" s="28" t="n">
         <v>0</v>
@@ -2377,32 +2401,34 @@
         <v>0</v>
       </c>
       <c r="F61" s="28" t="n">
-        <v>350</v>
-      </c>
-      <c r="G61" s="28" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G61" s="28" t="n">
+        <v>15174</v>
+      </c>
       <c r="H61" s="31" t="n">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="I61" s="31" t="n">
         <v>1</v>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Pay-per-lease fee PLACEHOLDER</t>
+          <t>Cancelled: last invoice 9/30/26. 2026: $15,174 for 1 lease. Enter a fee and mix here if renewed</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>All other / unknown</t>
+          <t>Apartment List</t>
         </is>
       </c>
       <c r="B62" s="29" t="n">
-        <v>0.053</v>
+        <v>0.018</v>
       </c>
       <c r="C62" s="29" t="n">
-        <v>0.042</v>
+        <v>0.083</v>
       </c>
       <c r="D62" s="28" t="n">
         <v>0</v>
@@ -2415,147 +2441,163 @@
       </c>
       <c r="G62" s="28" t="n"/>
       <c r="H62" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="I62" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>ACTUAL mix/conv. Not on ad tracker; enter pay-per-lease fee if charged</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>All other / unknown</t>
+        </is>
+      </c>
+      <c r="B63" s="29" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="C63" s="29" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="D63" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="28" t="n"/>
+      <c r="H63" s="31" t="n">
         <v>71</v>
       </c>
-      <c r="I62" s="31" t="n">
+      <c r="I63" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="J62" s="7" t="inlineStr">
-        <is>
-          <t>ACTUAL: sister community, RentCafe, walk-in, unknown, etc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>ACTUAL: sister community, RentCafe, walk-in, unknown, etc. (AptGeo $0 in 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>Total (lease mix must = 100%)</t>
         </is>
       </c>
-      <c r="B63" s="30">
-        <f>SUM(B54:B62)</f>
-        <v/>
-      </c>
-      <c r="C63" s="5">
-        <f>IF(ROUND(B63,4)=1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="H63" s="32">
-        <f>SUM(H54:H62)</f>
-        <v/>
-      </c>
-      <c r="I63" s="32">
-        <f>SUM(I54:I62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
+      <c r="B64" s="30">
+        <f>SUM(B55:B63)</f>
+        <v/>
+      </c>
+      <c r="C64" s="5">
+        <f>IF(ROUND(B64,4)=1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="H64" s="32">
+        <f>SUM(H55:H63)</f>
+        <v/>
+      </c>
+      <c r="I64" s="32">
+        <f>SUM(I55:I63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Leads per channel = leases from that channel ÷ its lead-to-lease rate. Shift the lease mix toward channels that convert to cut spend. Leave 2026 actual blank if unknown.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>Fixed &amp; program costs (property-level)</t>
         </is>
       </c>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="4" t="n"/>
-      <c r="E66" s="4" t="n"/>
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="4" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="16" t="inlineStr">
+      <c r="B67" s="4" t="n"/>
+      <c r="C67" s="4" t="n"/>
+      <c r="D67" s="4" t="n"/>
+      <c r="E67" s="4" t="n"/>
+      <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B67" s="16" t="inlineStr">
+      <c r="B68" s="16" t="inlineStr">
         <is>
           <t>Monthly ($)</t>
         </is>
       </c>
-      <c r="C67" s="16" t="inlineStr">
+      <c r="C68" s="16" t="inlineStr">
         <is>
           <t>One-time / annual ($)</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr"/>
-      <c r="E67" s="16" t="inlineStr"/>
-      <c r="F67" s="16" t="inlineStr"/>
-      <c r="G67" s="16" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr"/>
+      <c r="E68" s="16" t="inlineStr"/>
+      <c r="F68" s="16" t="inlineStr"/>
+      <c r="G68" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="25" t="inlineStr">
-        <is>
-          <t>CRM / lead management (allocated)</t>
-        </is>
-      </c>
-      <c r="B68" s="28" t="n">
-        <v>250</v>
-      </c>
-      <c r="C68" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: e.g. ~$1.50/unit/mo</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>AI leasing assistant / chat</t>
+          <t>CRM / lead management (allocated)</t>
         </is>
       </c>
       <c r="B69" s="28" t="n">
-        <v>166</v>
+        <v>250</v>
       </c>
       <c r="C69" s="28" t="n">
         <v>0</v>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: e.g. ~$1/unit/mo</t>
+          <t>PLACEHOLDER: e.g. ~$1.50/unit/mo</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>Reputation management / review software</t>
+          <t>AI leasing assistant / chat</t>
         </is>
       </c>
       <c r="B70" s="28" t="n">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="C70" s="28" t="n">
         <v>0</v>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>PLACEHOLDER: e.g. ~$1/unit/mo</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="25" t="inlineStr">
         <is>
-          <t>Website hosting &amp; maintenance</t>
+          <t>Reputation management / review software</t>
         </is>
       </c>
       <c r="B71" s="28" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C71" s="28" t="n">
         <v>0</v>
@@ -2569,50 +2611,50 @@
     <row r="72">
       <c r="A72" s="25" t="inlineStr">
         <is>
-          <t>Photography / video / virtual tour refresh</t>
+          <t>Website hosting &amp; maintenance</t>
         </is>
       </c>
       <c r="B72" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="C72" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="C72" s="28" t="n">
-        <v>1500</v>
-      </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: one-time 2027 refresh</t>
+          <t>PLACEHOLDER</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="25" t="inlineStr">
         <is>
-          <t>Signage &amp; banners</t>
+          <t>Photography / video / virtual tour refresh</t>
         </is>
       </c>
       <c r="B73" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C73" s="28" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>PLACEHOLDER: one-time 2027 refresh</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="25" t="inlineStr">
         <is>
-          <t>Print collateral</t>
+          <t>Signage &amp; banners</t>
         </is>
       </c>
       <c r="B74" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C74" s="28" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
@@ -2623,41 +2665,59 @@
     <row r="75">
       <c r="A75" s="25" t="inlineStr">
         <is>
-          <t>Resident events &amp; retention</t>
+          <t>Print collateral</t>
         </is>
       </c>
       <c r="B75" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C75" s="28" t="n">
-        <v>3000</v>
+        <v>300</v>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: ~4 events/yr; retention is cheaper than replacement</t>
+          <t>PLACEHOLDER</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="25" t="inlineStr">
         <is>
-          <t>Freelance / agency support</t>
+          <t>Resident events &amp; retention</t>
         </is>
       </c>
       <c r="B76" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C76" s="28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER: ~4 events/yr; retention is cheaper than replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="25" t="inlineStr">
+        <is>
+          <t>Freelance / agency support</t>
+        </is>
+      </c>
+      <c r="B77" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="C77" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
         <is>
           <t>Optional: outsourced help for a one-person team</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="G77" s="7" t="inlineStr">
+    <row r="78">
+      <c r="G78" s="7" t="inlineStr">
         <is>
           <t>One-time / annual amounts are spread evenly across 12 months in the Monthly Plan.</t>
         </is>
@@ -2805,51 +2865,51 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>Inputs!$B$38</f>
+        <f>Inputs!$B$39</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>Inputs!$B$39</f>
+        <f>Inputs!$B$40</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>Inputs!$B$40</f>
+        <f>Inputs!$B$41</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>Inputs!$B$41</f>
+        <f>Inputs!$B$42</f>
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>Inputs!$B$42</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$45</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>Inputs!$B$45</f>
+        <f>Inputs!$B$46</f>
         <v/>
       </c>
       <c r="J6" s="11">
-        <f>Inputs!$B$46</f>
+        <f>Inputs!$B$47</f>
         <v/>
       </c>
       <c r="K6" s="11">
-        <f>Inputs!$B$47</f>
+        <f>Inputs!$B$48</f>
         <v/>
       </c>
       <c r="L6" s="11">
-        <f>Inputs!$B$48</f>
+        <f>Inputs!$B$49</f>
         <v/>
       </c>
       <c r="M6" s="11">
-        <f>Inputs!$B$49</f>
+        <f>Inputs!$B$50</f>
         <v/>
       </c>
       <c r="N6" s="30">
@@ -3233,55 +3293,55 @@
     </row>
     <row r="14">
       <c r="A14" s="17">
-        <f>Inputs!$A$54</f>
+        <f>Inputs!$A$55</f>
         <v/>
       </c>
       <c r="B14" s="33">
-        <f>IFERROR(B12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(B12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="C14" s="33">
-        <f>IFERROR(C12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(C12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="D14" s="33">
-        <f>IFERROR(D12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(D12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="E14" s="33">
-        <f>IFERROR(E12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(E12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="F14" s="33">
-        <f>IFERROR(F12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(F12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="G14" s="33">
-        <f>IFERROR(G12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(G12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="H14" s="33">
-        <f>IFERROR(H12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(H12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="I14" s="33">
-        <f>IFERROR(I12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(I12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="J14" s="33">
-        <f>IFERROR(J12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(J12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="K14" s="33">
-        <f>IFERROR(K12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(K12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="L14" s="33">
-        <f>IFERROR(L12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(L12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="M14" s="33">
-        <f>IFERROR(M12*Inputs!$B$54/Inputs!$C$54,0)</f>
+        <f>IFERROR(M12*Inputs!$B$55/Inputs!$C$55,0)</f>
         <v/>
       </c>
       <c r="N14" s="34">
@@ -3291,55 +3351,55 @@
     </row>
     <row r="15">
       <c r="A15" s="17">
-        <f>Inputs!$A$55</f>
+        <f>Inputs!$A$56</f>
         <v/>
       </c>
       <c r="B15" s="33">
-        <f>IFERROR(B12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(B12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="C15" s="33">
-        <f>IFERROR(C12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(C12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="D15" s="33">
-        <f>IFERROR(D12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(D12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="E15" s="33">
-        <f>IFERROR(E12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(E12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="F15" s="33">
-        <f>IFERROR(F12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(F12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="G15" s="33">
-        <f>IFERROR(G12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(G12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="H15" s="33">
-        <f>IFERROR(H12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(H12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="I15" s="33">
-        <f>IFERROR(I12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(I12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="J15" s="33">
-        <f>IFERROR(J12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(J12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="K15" s="33">
-        <f>IFERROR(K12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(K12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="L15" s="33">
-        <f>IFERROR(L12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(L12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="M15" s="33">
-        <f>IFERROR(M12*Inputs!$B$55/Inputs!$C$55,0)</f>
+        <f>IFERROR(M12*Inputs!$B$56/Inputs!$C$56,0)</f>
         <v/>
       </c>
       <c r="N15" s="34">
@@ -3349,55 +3409,55 @@
     </row>
     <row r="16">
       <c r="A16" s="17">
-        <f>Inputs!$A$56</f>
+        <f>Inputs!$A$57</f>
         <v/>
       </c>
       <c r="B16" s="33">
-        <f>IFERROR(B12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(B12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="C16" s="33">
-        <f>IFERROR(C12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(C12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="D16" s="33">
-        <f>IFERROR(D12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(D12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="E16" s="33">
-        <f>IFERROR(E12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(E12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="F16" s="33">
-        <f>IFERROR(F12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(F12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="G16" s="33">
-        <f>IFERROR(G12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(G12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="H16" s="33">
-        <f>IFERROR(H12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(H12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="I16" s="33">
-        <f>IFERROR(I12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(I12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="J16" s="33">
-        <f>IFERROR(J12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(J12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="K16" s="33">
-        <f>IFERROR(K12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(K12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="L16" s="33">
-        <f>IFERROR(L12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(L12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="M16" s="33">
-        <f>IFERROR(M12*Inputs!$B$56/Inputs!$C$56,0)</f>
+        <f>IFERROR(M12*Inputs!$B$57/Inputs!$C$57,0)</f>
         <v/>
       </c>
       <c r="N16" s="34">
@@ -3407,55 +3467,55 @@
     </row>
     <row r="17">
       <c r="A17" s="17">
-        <f>Inputs!$A$57</f>
+        <f>Inputs!$A$58</f>
         <v/>
       </c>
       <c r="B17" s="33">
-        <f>IFERROR(B12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(B12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="C17" s="33">
-        <f>IFERROR(C12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(C12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="D17" s="33">
-        <f>IFERROR(D12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(D12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="E17" s="33">
-        <f>IFERROR(E12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(E12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="F17" s="33">
-        <f>IFERROR(F12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(F12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="G17" s="33">
-        <f>IFERROR(G12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(G12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="H17" s="33">
-        <f>IFERROR(H12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(H12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="I17" s="33">
-        <f>IFERROR(I12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(I12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="J17" s="33">
-        <f>IFERROR(J12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(J12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="K17" s="33">
-        <f>IFERROR(K12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(K12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="L17" s="33">
-        <f>IFERROR(L12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(L12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="M17" s="33">
-        <f>IFERROR(M12*Inputs!$B$57/Inputs!$C$57,0)</f>
+        <f>IFERROR(M12*Inputs!$B$58/Inputs!$C$58,0)</f>
         <v/>
       </c>
       <c r="N17" s="34">
@@ -3465,55 +3525,55 @@
     </row>
     <row r="18">
       <c r="A18" s="17">
-        <f>Inputs!$A$58</f>
+        <f>Inputs!$A$59</f>
         <v/>
       </c>
       <c r="B18" s="33">
-        <f>IFERROR(B12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(B12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="C18" s="33">
-        <f>IFERROR(C12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(C12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="D18" s="33">
-        <f>IFERROR(D12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(D12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="E18" s="33">
-        <f>IFERROR(E12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(E12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="F18" s="33">
-        <f>IFERROR(F12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(F12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="G18" s="33">
-        <f>IFERROR(G12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(G12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="H18" s="33">
-        <f>IFERROR(H12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(H12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="I18" s="33">
-        <f>IFERROR(I12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(I12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="J18" s="33">
-        <f>IFERROR(J12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(J12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="K18" s="33">
-        <f>IFERROR(K12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(K12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="L18" s="33">
-        <f>IFERROR(L12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(L12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="M18" s="33">
-        <f>IFERROR(M12*Inputs!$B$58/Inputs!$C$58,0)</f>
+        <f>IFERROR(M12*Inputs!$B$59/Inputs!$C$59,0)</f>
         <v/>
       </c>
       <c r="N18" s="34">
@@ -3523,55 +3583,55 @@
     </row>
     <row r="19">
       <c r="A19" s="17">
-        <f>Inputs!$A$59</f>
+        <f>Inputs!$A$60</f>
         <v/>
       </c>
       <c r="B19" s="33">
-        <f>IFERROR(B12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(B12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="C19" s="33">
-        <f>IFERROR(C12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(C12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="D19" s="33">
-        <f>IFERROR(D12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(D12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="E19" s="33">
-        <f>IFERROR(E12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(E12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="F19" s="33">
-        <f>IFERROR(F12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(F12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="G19" s="33">
-        <f>IFERROR(G12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(G12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="H19" s="33">
-        <f>IFERROR(H12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(H12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="I19" s="33">
-        <f>IFERROR(I12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(I12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="J19" s="33">
-        <f>IFERROR(J12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(J12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="K19" s="33">
-        <f>IFERROR(K12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(K12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="L19" s="33">
-        <f>IFERROR(L12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(L12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="M19" s="33">
-        <f>IFERROR(M12*Inputs!$B$59/Inputs!$C$59,0)</f>
+        <f>IFERROR(M12*Inputs!$B$60/Inputs!$C$60,0)</f>
         <v/>
       </c>
       <c r="N19" s="34">
@@ -3581,55 +3641,55 @@
     </row>
     <row r="20">
       <c r="A20" s="17">
-        <f>Inputs!$A$60</f>
+        <f>Inputs!$A$61</f>
         <v/>
       </c>
       <c r="B20" s="33">
-        <f>IFERROR(B12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(B12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="C20" s="33">
-        <f>IFERROR(C12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(C12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="D20" s="33">
-        <f>IFERROR(D12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(D12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="E20" s="33">
-        <f>IFERROR(E12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(E12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="F20" s="33">
-        <f>IFERROR(F12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(F12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="G20" s="33">
-        <f>IFERROR(G12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(G12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="H20" s="33">
-        <f>IFERROR(H12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(H12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="I20" s="33">
-        <f>IFERROR(I12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(I12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="J20" s="33">
-        <f>IFERROR(J12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(J12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="K20" s="33">
-        <f>IFERROR(K12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(K12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="L20" s="33">
-        <f>IFERROR(L12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(L12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="M20" s="33">
-        <f>IFERROR(M12*Inputs!$B$60/Inputs!$C$60,0)</f>
+        <f>IFERROR(M12*Inputs!$B$61/Inputs!$C$61,0)</f>
         <v/>
       </c>
       <c r="N20" s="34">
@@ -3639,55 +3699,55 @@
     </row>
     <row r="21">
       <c r="A21" s="17">
-        <f>Inputs!$A$61</f>
+        <f>Inputs!$A$62</f>
         <v/>
       </c>
       <c r="B21" s="33">
-        <f>IFERROR(B12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(B12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="C21" s="33">
-        <f>IFERROR(C12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(C12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="D21" s="33">
-        <f>IFERROR(D12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(D12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="E21" s="33">
-        <f>IFERROR(E12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(E12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="F21" s="33">
-        <f>IFERROR(F12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(F12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="G21" s="33">
-        <f>IFERROR(G12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(G12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="H21" s="33">
-        <f>IFERROR(H12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(H12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="I21" s="33">
-        <f>IFERROR(I12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(I12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="J21" s="33">
-        <f>IFERROR(J12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(J12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="K21" s="33">
-        <f>IFERROR(K12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(K12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="L21" s="33">
-        <f>IFERROR(L12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(L12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="M21" s="33">
-        <f>IFERROR(M12*Inputs!$B$61/Inputs!$C$61,0)</f>
+        <f>IFERROR(M12*Inputs!$B$62/Inputs!$C$62,0)</f>
         <v/>
       </c>
       <c r="N21" s="34">
@@ -3697,55 +3757,55 @@
     </row>
     <row r="22">
       <c r="A22" s="17">
-        <f>Inputs!$A$62</f>
+        <f>Inputs!$A$63</f>
         <v/>
       </c>
       <c r="B22" s="33">
-        <f>IFERROR(B12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(B12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="C22" s="33">
-        <f>IFERROR(C12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(C12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="D22" s="33">
-        <f>IFERROR(D12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(D12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="E22" s="33">
-        <f>IFERROR(E12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(E12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="F22" s="33">
-        <f>IFERROR(F12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(F12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="G22" s="33">
-        <f>IFERROR(G12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(G12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="H22" s="33">
-        <f>IFERROR(H12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(H12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="I22" s="33">
-        <f>IFERROR(I12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(I12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="J22" s="33">
-        <f>IFERROR(J12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(J12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="K22" s="33">
-        <f>IFERROR(K12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(K12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="L22" s="33">
-        <f>IFERROR(L12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(L12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="M22" s="33">
-        <f>IFERROR(M12*Inputs!$B$62/Inputs!$C$62,0)</f>
+        <f>IFERROR(M12*Inputs!$B$63/Inputs!$C$63,0)</f>
         <v/>
       </c>
       <c r="N22" s="34">
@@ -3972,55 +4032,55 @@
     </row>
     <row r="28">
       <c r="A28" s="17">
-        <f>Inputs!$A$54</f>
+        <f>Inputs!$A$55</f>
         <v/>
       </c>
       <c r="B28" s="37">
-        <f>Inputs!$E$54+B14*Inputs!$D$54+B12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+B14*Inputs!$D$55+B12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="C28" s="37">
-        <f>Inputs!$E$54+C14*Inputs!$D$54+C12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+C14*Inputs!$D$55+C12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="D28" s="37">
-        <f>Inputs!$E$54+D14*Inputs!$D$54+D12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+D14*Inputs!$D$55+D12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="E28" s="37">
-        <f>Inputs!$E$54+E14*Inputs!$D$54+E12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+E14*Inputs!$D$55+E12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="F28" s="37">
-        <f>Inputs!$E$54+F14*Inputs!$D$54+F12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+F14*Inputs!$D$55+F12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="G28" s="37">
-        <f>Inputs!$E$54+G14*Inputs!$D$54+G12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+G14*Inputs!$D$55+G12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="H28" s="37">
-        <f>Inputs!$E$54+H14*Inputs!$D$54+H12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+H14*Inputs!$D$55+H12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="I28" s="37">
-        <f>Inputs!$E$54+I14*Inputs!$D$54+I12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+I14*Inputs!$D$55+I12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="J28" s="37">
-        <f>Inputs!$E$54+J14*Inputs!$D$54+J12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+J14*Inputs!$D$55+J12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="K28" s="37">
-        <f>Inputs!$E$54+K14*Inputs!$D$54+K12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+K14*Inputs!$D$55+K12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="L28" s="37">
-        <f>Inputs!$E$54+L14*Inputs!$D$54+L12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+L14*Inputs!$D$55+L12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="M28" s="37">
-        <f>Inputs!$E$54+M14*Inputs!$D$54+M12*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+M14*Inputs!$D$55+M12*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="N28" s="38">
@@ -4030,55 +4090,55 @@
     </row>
     <row r="29">
       <c r="A29" s="17">
-        <f>Inputs!$A$55</f>
+        <f>Inputs!$A$56</f>
         <v/>
       </c>
       <c r="B29" s="37">
-        <f>Inputs!$E$55+B15*Inputs!$D$55+B12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+B15*Inputs!$D$56+B12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="C29" s="37">
-        <f>Inputs!$E$55+C15*Inputs!$D$55+C12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+C15*Inputs!$D$56+C12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="D29" s="37">
-        <f>Inputs!$E$55+D15*Inputs!$D$55+D12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+D15*Inputs!$D$56+D12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="E29" s="37">
-        <f>Inputs!$E$55+E15*Inputs!$D$55+E12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+E15*Inputs!$D$56+E12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="F29" s="37">
-        <f>Inputs!$E$55+F15*Inputs!$D$55+F12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+F15*Inputs!$D$56+F12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="G29" s="37">
-        <f>Inputs!$E$55+G15*Inputs!$D$55+G12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+G15*Inputs!$D$56+G12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="H29" s="37">
-        <f>Inputs!$E$55+H15*Inputs!$D$55+H12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+H15*Inputs!$D$56+H12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="I29" s="37">
-        <f>Inputs!$E$55+I15*Inputs!$D$55+I12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+I15*Inputs!$D$56+I12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="J29" s="37">
-        <f>Inputs!$E$55+J15*Inputs!$D$55+J12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+J15*Inputs!$D$56+J12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="K29" s="37">
-        <f>Inputs!$E$55+K15*Inputs!$D$55+K12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+K15*Inputs!$D$56+K12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="L29" s="37">
-        <f>Inputs!$E$55+L15*Inputs!$D$55+L12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+L15*Inputs!$D$56+L12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="M29" s="37">
-        <f>Inputs!$E$55+M15*Inputs!$D$55+M12*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+M15*Inputs!$D$56+M12*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="N29" s="38">
@@ -4088,55 +4148,55 @@
     </row>
     <row r="30">
       <c r="A30" s="17">
-        <f>Inputs!$A$56</f>
+        <f>Inputs!$A$57</f>
         <v/>
       </c>
       <c r="B30" s="37">
-        <f>Inputs!$E$56+B16*Inputs!$D$56+B12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+B16*Inputs!$D$57+B12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="C30" s="37">
-        <f>Inputs!$E$56+C16*Inputs!$D$56+C12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+C16*Inputs!$D$57+C12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="D30" s="37">
-        <f>Inputs!$E$56+D16*Inputs!$D$56+D12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+D16*Inputs!$D$57+D12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="E30" s="37">
-        <f>Inputs!$E$56+E16*Inputs!$D$56+E12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+E16*Inputs!$D$57+E12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="F30" s="37">
-        <f>Inputs!$E$56+F16*Inputs!$D$56+F12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+F16*Inputs!$D$57+F12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="G30" s="37">
-        <f>Inputs!$E$56+G16*Inputs!$D$56+G12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+G16*Inputs!$D$57+G12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="H30" s="37">
-        <f>Inputs!$E$56+H16*Inputs!$D$56+H12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+H16*Inputs!$D$57+H12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="I30" s="37">
-        <f>Inputs!$E$56+I16*Inputs!$D$56+I12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+I16*Inputs!$D$57+I12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="J30" s="37">
-        <f>Inputs!$E$56+J16*Inputs!$D$56+J12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+J16*Inputs!$D$57+J12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="K30" s="37">
-        <f>Inputs!$E$56+K16*Inputs!$D$56+K12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+K16*Inputs!$D$57+K12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="L30" s="37">
-        <f>Inputs!$E$56+L16*Inputs!$D$56+L12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+L16*Inputs!$D$57+L12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="M30" s="37">
-        <f>Inputs!$E$56+M16*Inputs!$D$56+M12*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+M16*Inputs!$D$57+M12*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="N30" s="38">
@@ -4146,55 +4206,55 @@
     </row>
     <row r="31">
       <c r="A31" s="17">
-        <f>Inputs!$A$57</f>
+        <f>Inputs!$A$58</f>
         <v/>
       </c>
       <c r="B31" s="37">
-        <f>Inputs!$E$57+B17*Inputs!$D$57+B12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+B17*Inputs!$D$58+B12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="C31" s="37">
-        <f>Inputs!$E$57+C17*Inputs!$D$57+C12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+C17*Inputs!$D$58+C12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="D31" s="37">
-        <f>Inputs!$E$57+D17*Inputs!$D$57+D12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+D17*Inputs!$D$58+D12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="E31" s="37">
-        <f>Inputs!$E$57+E17*Inputs!$D$57+E12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+E17*Inputs!$D$58+E12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="F31" s="37">
-        <f>Inputs!$E$57+F17*Inputs!$D$57+F12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+F17*Inputs!$D$58+F12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="G31" s="37">
-        <f>Inputs!$E$57+G17*Inputs!$D$57+G12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+G17*Inputs!$D$58+G12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="H31" s="37">
-        <f>Inputs!$E$57+H17*Inputs!$D$57+H12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+H17*Inputs!$D$58+H12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="I31" s="37">
-        <f>Inputs!$E$57+I17*Inputs!$D$57+I12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+I17*Inputs!$D$58+I12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="J31" s="37">
-        <f>Inputs!$E$57+J17*Inputs!$D$57+J12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+J17*Inputs!$D$58+J12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="K31" s="37">
-        <f>Inputs!$E$57+K17*Inputs!$D$57+K12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+K17*Inputs!$D$58+K12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="L31" s="37">
-        <f>Inputs!$E$57+L17*Inputs!$D$57+L12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+L17*Inputs!$D$58+L12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="M31" s="37">
-        <f>Inputs!$E$57+M17*Inputs!$D$57+M12*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+M17*Inputs!$D$58+M12*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="N31" s="38">
@@ -4204,55 +4264,55 @@
     </row>
     <row r="32">
       <c r="A32" s="17">
-        <f>Inputs!$A$58</f>
+        <f>Inputs!$A$59</f>
         <v/>
       </c>
       <c r="B32" s="37">
-        <f>Inputs!$E$58+B18*Inputs!$D$58+B12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+B18*Inputs!$D$59+B12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="C32" s="37">
-        <f>Inputs!$E$58+C18*Inputs!$D$58+C12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+C18*Inputs!$D$59+C12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="D32" s="37">
-        <f>Inputs!$E$58+D18*Inputs!$D$58+D12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+D18*Inputs!$D$59+D12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="E32" s="37">
-        <f>Inputs!$E$58+E18*Inputs!$D$58+E12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+E18*Inputs!$D$59+E12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="F32" s="37">
-        <f>Inputs!$E$58+F18*Inputs!$D$58+F12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+F18*Inputs!$D$59+F12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="G32" s="37">
-        <f>Inputs!$E$58+G18*Inputs!$D$58+G12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+G18*Inputs!$D$59+G12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="H32" s="37">
-        <f>Inputs!$E$58+H18*Inputs!$D$58+H12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+H18*Inputs!$D$59+H12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="I32" s="37">
-        <f>Inputs!$E$58+I18*Inputs!$D$58+I12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+I18*Inputs!$D$59+I12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="J32" s="37">
-        <f>Inputs!$E$58+J18*Inputs!$D$58+J12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+J18*Inputs!$D$59+J12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="K32" s="37">
-        <f>Inputs!$E$58+K18*Inputs!$D$58+K12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+K18*Inputs!$D$59+K12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="L32" s="37">
-        <f>Inputs!$E$58+L18*Inputs!$D$58+L12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+L18*Inputs!$D$59+L12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="M32" s="37">
-        <f>Inputs!$E$58+M18*Inputs!$D$58+M12*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+M18*Inputs!$D$59+M12*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="N32" s="38">
@@ -4262,55 +4322,55 @@
     </row>
     <row r="33">
       <c r="A33" s="17">
-        <f>Inputs!$A$59</f>
+        <f>Inputs!$A$60</f>
         <v/>
       </c>
       <c r="B33" s="37">
-        <f>Inputs!$E$59+B19*Inputs!$D$59+B12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+B19*Inputs!$D$60+B12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="C33" s="37">
-        <f>Inputs!$E$59+C19*Inputs!$D$59+C12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+C19*Inputs!$D$60+C12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="D33" s="37">
-        <f>Inputs!$E$59+D19*Inputs!$D$59+D12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+D19*Inputs!$D$60+D12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="E33" s="37">
-        <f>Inputs!$E$59+E19*Inputs!$D$59+E12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+E19*Inputs!$D$60+E12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="F33" s="37">
-        <f>Inputs!$E$59+F19*Inputs!$D$59+F12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+F19*Inputs!$D$60+F12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="G33" s="37">
-        <f>Inputs!$E$59+G19*Inputs!$D$59+G12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+G19*Inputs!$D$60+G12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="H33" s="37">
-        <f>Inputs!$E$59+H19*Inputs!$D$59+H12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+H19*Inputs!$D$60+H12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="I33" s="37">
-        <f>Inputs!$E$59+I19*Inputs!$D$59+I12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+I19*Inputs!$D$60+I12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="J33" s="37">
-        <f>Inputs!$E$59+J19*Inputs!$D$59+J12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+J19*Inputs!$D$60+J12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="K33" s="37">
-        <f>Inputs!$E$59+K19*Inputs!$D$59+K12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+K19*Inputs!$D$60+K12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="L33" s="37">
-        <f>Inputs!$E$59+L19*Inputs!$D$59+L12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+L19*Inputs!$D$60+L12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="M33" s="37">
-        <f>Inputs!$E$59+M19*Inputs!$D$59+M12*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+M19*Inputs!$D$60+M12*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="N33" s="38">
@@ -4320,55 +4380,55 @@
     </row>
     <row r="34">
       <c r="A34" s="17">
-        <f>Inputs!$A$60</f>
+        <f>Inputs!$A$61</f>
         <v/>
       </c>
       <c r="B34" s="37">
-        <f>Inputs!$E$60+B20*Inputs!$D$60+B12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+B20*Inputs!$D$61+B12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="C34" s="37">
-        <f>Inputs!$E$60+C20*Inputs!$D$60+C12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+C20*Inputs!$D$61+C12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="D34" s="37">
-        <f>Inputs!$E$60+D20*Inputs!$D$60+D12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+D20*Inputs!$D$61+D12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="E34" s="37">
-        <f>Inputs!$E$60+E20*Inputs!$D$60+E12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+E20*Inputs!$D$61+E12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="F34" s="37">
-        <f>Inputs!$E$60+F20*Inputs!$D$60+F12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+F20*Inputs!$D$61+F12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="G34" s="37">
-        <f>Inputs!$E$60+G20*Inputs!$D$60+G12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+G20*Inputs!$D$61+G12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="H34" s="37">
-        <f>Inputs!$E$60+H20*Inputs!$D$60+H12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+H20*Inputs!$D$61+H12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="I34" s="37">
-        <f>Inputs!$E$60+I20*Inputs!$D$60+I12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+I20*Inputs!$D$61+I12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="J34" s="37">
-        <f>Inputs!$E$60+J20*Inputs!$D$60+J12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+J20*Inputs!$D$61+J12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="K34" s="37">
-        <f>Inputs!$E$60+K20*Inputs!$D$60+K12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+K20*Inputs!$D$61+K12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="L34" s="37">
-        <f>Inputs!$E$60+L20*Inputs!$D$60+L12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+L20*Inputs!$D$61+L12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="M34" s="37">
-        <f>Inputs!$E$60+M20*Inputs!$D$60+M12*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+M20*Inputs!$D$61+M12*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="N34" s="38">
@@ -4378,55 +4438,55 @@
     </row>
     <row r="35">
       <c r="A35" s="17">
-        <f>Inputs!$A$61</f>
+        <f>Inputs!$A$62</f>
         <v/>
       </c>
       <c r="B35" s="37">
-        <f>Inputs!$E$61+B21*Inputs!$D$61+B12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+B21*Inputs!$D$62+B12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="C35" s="37">
-        <f>Inputs!$E$61+C21*Inputs!$D$61+C12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+C21*Inputs!$D$62+C12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="D35" s="37">
-        <f>Inputs!$E$61+D21*Inputs!$D$61+D12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+D21*Inputs!$D$62+D12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="E35" s="37">
-        <f>Inputs!$E$61+E21*Inputs!$D$61+E12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+E21*Inputs!$D$62+E12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="F35" s="37">
-        <f>Inputs!$E$61+F21*Inputs!$D$61+F12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+F21*Inputs!$D$62+F12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="G35" s="37">
-        <f>Inputs!$E$61+G21*Inputs!$D$61+G12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+G21*Inputs!$D$62+G12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="H35" s="37">
-        <f>Inputs!$E$61+H21*Inputs!$D$61+H12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+H21*Inputs!$D$62+H12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="I35" s="37">
-        <f>Inputs!$E$61+I21*Inputs!$D$61+I12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+I21*Inputs!$D$62+I12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="J35" s="37">
-        <f>Inputs!$E$61+J21*Inputs!$D$61+J12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+J21*Inputs!$D$62+J12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="K35" s="37">
-        <f>Inputs!$E$61+K21*Inputs!$D$61+K12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+K21*Inputs!$D$62+K12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="L35" s="37">
-        <f>Inputs!$E$61+L21*Inputs!$D$61+L12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+L21*Inputs!$D$62+L12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="M35" s="37">
-        <f>Inputs!$E$61+M21*Inputs!$D$61+M12*Inputs!$B$61*Inputs!$F$61</f>
+        <f>Inputs!$E$62+M21*Inputs!$D$62+M12*Inputs!$B$62*Inputs!$F$62</f>
         <v/>
       </c>
       <c r="N35" s="38">
@@ -4436,55 +4496,55 @@
     </row>
     <row r="36">
       <c r="A36" s="17">
-        <f>Inputs!$A$62</f>
+        <f>Inputs!$A$63</f>
         <v/>
       </c>
       <c r="B36" s="37">
-        <f>Inputs!$E$62+B22*Inputs!$D$62+B12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+B22*Inputs!$D$63+B12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="C36" s="37">
-        <f>Inputs!$E$62+C22*Inputs!$D$62+C12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+C22*Inputs!$D$63+C12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="D36" s="37">
-        <f>Inputs!$E$62+D22*Inputs!$D$62+D12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+D22*Inputs!$D$63+D12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="E36" s="37">
-        <f>Inputs!$E$62+E22*Inputs!$D$62+E12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+E22*Inputs!$D$63+E12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="F36" s="37">
-        <f>Inputs!$E$62+F22*Inputs!$D$62+F12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+F22*Inputs!$D$63+F12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="G36" s="37">
-        <f>Inputs!$E$62+G22*Inputs!$D$62+G12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+G22*Inputs!$D$63+G12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="H36" s="37">
-        <f>Inputs!$E$62+H22*Inputs!$D$62+H12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+H22*Inputs!$D$63+H12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="I36" s="37">
-        <f>Inputs!$E$62+I22*Inputs!$D$62+I12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+I22*Inputs!$D$63+I12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="J36" s="37">
-        <f>Inputs!$E$62+J22*Inputs!$D$62+J12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+J22*Inputs!$D$63+J12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="K36" s="37">
-        <f>Inputs!$E$62+K22*Inputs!$D$62+K12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+K22*Inputs!$D$63+K12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="L36" s="37">
-        <f>Inputs!$E$62+L22*Inputs!$D$62+L12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+L22*Inputs!$D$63+L12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="M36" s="37">
-        <f>Inputs!$E$62+M22*Inputs!$D$62+M12*Inputs!$B$62*Inputs!$F$62</f>
+        <f>Inputs!$E$63+M22*Inputs!$D$63+M12*Inputs!$B$63*Inputs!$F$63</f>
         <v/>
       </c>
       <c r="N36" s="38">
@@ -4573,55 +4633,55 @@
     </row>
     <row r="39">
       <c r="A39" s="17">
-        <f>Inputs!$A$68</f>
+        <f>Inputs!$A$69</f>
         <v/>
       </c>
       <c r="B39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="C39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="D39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="E39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="F39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="G39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="H39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="I39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="J39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="K39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="L39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="M39" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="N39" s="38">
@@ -4631,55 +4691,55 @@
     </row>
     <row r="40">
       <c r="A40" s="17">
-        <f>Inputs!$A$69</f>
+        <f>Inputs!$A$70</f>
         <v/>
       </c>
       <c r="B40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="C40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="D40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="E40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="F40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="G40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="H40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="I40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="J40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="K40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="L40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="M40" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="N40" s="38">
@@ -4689,55 +4749,55 @@
     </row>
     <row r="41">
       <c r="A41" s="17">
-        <f>Inputs!$A$70</f>
+        <f>Inputs!$A$71</f>
         <v/>
       </c>
       <c r="B41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="C41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="D41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="E41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="F41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="G41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="H41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="I41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="J41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="K41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="L41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="M41" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="N41" s="38">
@@ -4747,55 +4807,55 @@
     </row>
     <row r="42">
       <c r="A42" s="17">
-        <f>Inputs!$A$71</f>
+        <f>Inputs!$A$72</f>
         <v/>
       </c>
       <c r="B42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="C42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="D42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="E42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="F42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="G42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="H42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="I42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="J42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="K42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="L42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="M42" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="N42" s="38">
@@ -4805,55 +4865,55 @@
     </row>
     <row r="43">
       <c r="A43" s="17">
-        <f>Inputs!$A$72</f>
+        <f>Inputs!$A$73</f>
         <v/>
       </c>
       <c r="B43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="C43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="D43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="E43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="F43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="G43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="H43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="I43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="J43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="K43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="L43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="M43" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="N43" s="38">
@@ -4863,55 +4923,55 @@
     </row>
     <row r="44">
       <c r="A44" s="17">
-        <f>Inputs!$A$73</f>
+        <f>Inputs!$A$74</f>
         <v/>
       </c>
       <c r="B44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="C44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="D44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="E44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="F44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="G44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="H44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="I44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="J44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="K44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="L44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="M44" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="N44" s="38">
@@ -4921,55 +4981,55 @@
     </row>
     <row r="45">
       <c r="A45" s="17">
-        <f>Inputs!$A$74</f>
+        <f>Inputs!$A$75</f>
         <v/>
       </c>
       <c r="B45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="C45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="D45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="E45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="F45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="G45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="H45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="I45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="J45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="K45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="L45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="M45" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>Inputs!$B$75+Inputs!$C$75/12</f>
         <v/>
       </c>
       <c r="N45" s="38">
@@ -4979,55 +5039,55 @@
     </row>
     <row r="46">
       <c r="A46" s="17">
-        <f>Inputs!$A$75</f>
+        <f>Inputs!$A$76</f>
         <v/>
       </c>
       <c r="B46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="C46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="D46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="E46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="F46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="G46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="H46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="I46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="J46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="K46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="L46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="M46" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+        <f>Inputs!$B$76+Inputs!$C$76/12</f>
         <v/>
       </c>
       <c r="N46" s="38">
@@ -5037,55 +5097,55 @@
     </row>
     <row r="47">
       <c r="A47" s="17">
-        <f>Inputs!$A$76</f>
+        <f>Inputs!$A$77</f>
         <v/>
       </c>
       <c r="B47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="C47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="D47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="E47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="F47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="G47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="H47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="I47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="J47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="K47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="L47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="M47" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
+        <f>Inputs!$B$77+Inputs!$C$77/12</f>
         <v/>
       </c>
       <c r="N47" s="38">
@@ -5297,51 +5357,51 @@
         </is>
       </c>
       <c r="B52" s="37">
-        <f>B51*Inputs!$B$33</f>
+        <f>B51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="C52" s="37">
-        <f>C51*Inputs!$B$33</f>
+        <f>C51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="D52" s="37">
-        <f>D51*Inputs!$B$33</f>
+        <f>D51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="E52" s="37">
-        <f>E51*Inputs!$B$33</f>
+        <f>E51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="F52" s="37">
-        <f>F51*Inputs!$B$33</f>
+        <f>F51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="G52" s="37">
-        <f>G51*Inputs!$B$33</f>
+        <f>G51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="H52" s="37">
-        <f>H51*Inputs!$B$33</f>
+        <f>H51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="I52" s="37">
-        <f>I51*Inputs!$B$33</f>
+        <f>I51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="J52" s="37">
-        <f>J51*Inputs!$B$33</f>
+        <f>J51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="K52" s="37">
-        <f>K51*Inputs!$B$33</f>
+        <f>K51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="L52" s="37">
-        <f>L51*Inputs!$B$33</f>
+        <f>L51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="M52" s="37">
-        <f>M51*Inputs!$B$33</f>
+        <f>M51*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="N52" s="38">
@@ -5419,7 +5479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5531,36 +5591,43 @@
     <row r="18">
       <c r="A18" s="40" t="inlineStr">
         <is>
-          <t>2. Invoices / contracts: Zillow, Apartments.com, Rently, PPC, Apartment List, MLS, software; note 2027 renewal pricing.</t>
+          <t>Done from the 2026 Ad Spend Tracking sheet: Digible, Zillow, CoStar (cancelled 9/30/26), AptGeo and website spend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="40" t="inlineStr">
         <is>
-          <t>3. 2026 actual marketing spend by channel (for the variance column).</t>
+          <t>2. 2027 price changes from Digible and Zillow; whether Rently, MLS or Apartment List are billed somewhere else.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="40" t="inlineStr">
         <is>
+          <t>3. Digible's lead and lease attribution report (WAR may credit their ads to Property Website).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
           <t>4. Fixed-cost items: CRM, AI leasing, reputation, website, photography, signage, events.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="40" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="40" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
         <is>
           <t>Rolling out to the portfolio</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="40" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>Copy this workbook once per property (or duplicate the Inputs tab) and change the Inputs. Prosper 207 is in lease-up and needs a separate lease-up model (absorption pace, not turnover).</t>
         </is>

</xml_diff>

<commit_message>
Add MLS fee; exclude Rently and CRM costs; fold Apartment List into other
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S4EZy9r3vcic7sA8Y6yuUD
</commit_message>
<xml_diff>
--- a/Harrison_Landing_2027_Marketing_Budget.xlsx
+++ b/Harrison_Landing_2027_Marketing_Budget.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>'Monthly Plan'!$N$52</f>
+        <f>'Monthly Plan'!$N$49</f>
         <v/>
       </c>
       <c r="E5" s="7" t="inlineStr"/>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>'Monthly Plan'!$N$36</f>
+        <f>'Monthly Plan'!$N$34</f>
         <v/>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>IFERROR(B17/'Monthly Plan'!$N$22,0)</f>
+        <f>IFERROR(B17/'Monthly Plan'!$N$21,0)</f>
         <v/>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B19" s="13">
-        <f>'Monthly Plan'!$N$22</f>
+        <f>'Monthly Plan'!$N$21</f>
         <v/>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>'Monthly Plan'!$N$24</f>
+        <f>'Monthly Plan'!$N$23</f>
         <v/>
       </c>
       <c r="E20" s="7" t="inlineStr"/>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>IFERROR('Monthly Plan'!$N$36/B19,0)</f>
+        <f>IFERROR('Monthly Plan'!$N$34/B19,0)</f>
         <v/>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1002,7 +1002,7 @@
         <v/>
       </c>
       <c r="B38" s="9">
-        <f>'Monthly Plan'!$N$27</f>
+        <f>'Monthly Plan'!$N$26</f>
         <v/>
       </c>
       <c r="C38" s="9">
@@ -1036,7 +1036,7 @@
         <v/>
       </c>
       <c r="B39" s="9">
-        <f>'Monthly Plan'!$N$28</f>
+        <f>'Monthly Plan'!$N$27</f>
         <v/>
       </c>
       <c r="C39" s="9">
@@ -1070,7 +1070,7 @@
         <v/>
       </c>
       <c r="B40" s="9">
-        <f>'Monthly Plan'!$N$29</f>
+        <f>'Monthly Plan'!$N$28</f>
         <v/>
       </c>
       <c r="C40" s="9">
@@ -1104,7 +1104,7 @@
         <v/>
       </c>
       <c r="B41" s="9">
-        <f>'Monthly Plan'!$N$30</f>
+        <f>'Monthly Plan'!$N$29</f>
         <v/>
       </c>
       <c r="C41" s="9">
@@ -1138,7 +1138,7 @@
         <v/>
       </c>
       <c r="B42" s="9">
-        <f>'Monthly Plan'!$N$31</f>
+        <f>'Monthly Plan'!$N$30</f>
         <v/>
       </c>
       <c r="C42" s="9">
@@ -1172,7 +1172,7 @@
         <v/>
       </c>
       <c r="B43" s="9">
-        <f>'Monthly Plan'!$N$32</f>
+        <f>'Monthly Plan'!$N$31</f>
         <v/>
       </c>
       <c r="C43" s="9">
@@ -1206,7 +1206,7 @@
         <v/>
       </c>
       <c r="B44" s="9">
-        <f>'Monthly Plan'!$N$33</f>
+        <f>'Monthly Plan'!$N$32</f>
         <v/>
       </c>
       <c r="C44" s="9">
@@ -1240,7 +1240,7 @@
         <v/>
       </c>
       <c r="B45" s="9">
-        <f>'Monthly Plan'!$N$34</f>
+        <f>'Monthly Plan'!$N$33</f>
         <v/>
       </c>
       <c r="C45" s="9">
@@ -1269,43 +1269,24 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="17">
-        <f>Inputs!$A$62</f>
-        <v/>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Fixed, program &amp; retention costs</t>
+        </is>
       </c>
       <c r="B46" s="9">
-        <f>'Monthly Plan'!$N$35</f>
-        <v/>
-      </c>
-      <c r="C46" s="9">
-        <f>IF(Inputs!$G$62="","",Inputs!$G$62)</f>
-        <v/>
-      </c>
-      <c r="D46" s="18">
-        <f>IF(C46="","",B46-C46)</f>
+        <f>'Monthly Plan'!$N$45</f>
         <v/>
       </c>
       <c r="E46" s="19">
         <f>IFERROR(B46/B5,0)</f>
         <v/>
       </c>
-      <c r="F46" s="12">
-        <f>'Monthly Plan'!$N$21</f>
-        <v/>
-      </c>
-      <c r="G46" s="20">
-        <f>B17*Inputs!$B$62</f>
-        <v/>
-      </c>
-      <c r="H46" s="18">
-        <f>IFERROR(B46/G46,0)</f>
-        <v/>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Fixed, program &amp; retention costs</t>
+          <t>Contingency</t>
         </is>
       </c>
       <c r="B47" s="9">
@@ -1318,59 +1299,44 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B48" s="9">
-        <f>'Monthly Plan'!$N$51</f>
-        <v/>
-      </c>
-      <c r="E48" s="19">
-        <f>IFERROR(B48/B5,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="21" t="inlineStr">
+      <c r="A48" s="21" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B49" s="22">
-        <f>SUM(B38:B48)</f>
-        <v/>
-      </c>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="23" t="n"/>
-      <c r="E49" s="24">
-        <f>SUM(E38:E48)</f>
-        <v/>
-      </c>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="23" t="n"/>
-      <c r="H49" s="23" t="n"/>
+      <c r="B48" s="22">
+        <f>SUM(B38:B47)</f>
+        <v/>
+      </c>
+      <c r="C48" s="23" t="n"/>
+      <c r="D48" s="23" t="n"/>
+      <c r="E48" s="24">
+        <f>SUM(E38:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="23" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Input checks</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Input checks</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Channel lease mix sums to 100%</t>
         </is>
       </c>
-      <c r="B52" s="17">
-        <f>Inputs!$C$63</f>
+      <c r="B51" s="17">
+        <f>Inputs!$C$62</f>
         <v/>
       </c>
     </row>
@@ -1385,7 +1351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2348,7 +2314,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Mix/conv ACTUAL (WAR T-12). Fee ACTUAL: $958/mo since Oct 2026 (was $930). Mix includes Apts.com's former share</t>
+          <t>Mix/conv ACTUAL (WAR T-12). Fee ACTUAL: $958/mo is the 2027 rate (updated Oct 2026). Mix includes Apts.com's former share</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2370,7 @@
         <v>0</v>
       </c>
       <c r="E56" s="28" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F56" s="28" t="n">
         <v>0</v>
@@ -2418,7 +2384,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Not on ad tracker: any MLS / agent fees?</t>
+          <t>Mix/conv ACTUAL (WAR T-12). Fee ACTUAL: $1,000/mo for one listing (fixed, per user)</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2452,7 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Not on ad tracker: confirm if billed elsewhere</t>
+          <t>ACTUAL mix/conv. Cost excluded from this budget (per user)</t>
         </is>
       </c>
     </row>
@@ -2565,14 +2531,14 @@
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>Apartment List</t>
+          <t>All other / unknown</t>
         </is>
       </c>
       <c r="B61" s="29" t="n">
-        <v>0.018</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="C61" s="29" t="n">
-        <v>0.083</v>
+        <v>0.048</v>
       </c>
       <c r="D61" s="28" t="n">
         <v>0</v>
@@ -2585,184 +2551,168 @@
       </c>
       <c r="G61" s="28" t="n"/>
       <c r="H61" s="31" t="n">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="I61" s="31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>ACTUAL mix/conv. Not on ad tracker; enter pay-per-lease fee if charged</t>
+          <t>ACTUAL: Apartment List, sister community, RentCafe, walk-in, unknown, etc. (AptGeo $0 in 2026)</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="25" t="inlineStr">
-        <is>
-          <t>All other / unknown</t>
-        </is>
-      </c>
-      <c r="B62" s="29" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="C62" s="29" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="D62" s="28" t="n">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Total (lease mix must = 100%)</t>
+        </is>
+      </c>
+      <c r="B62" s="30">
+        <f>SUM(B54:B61)</f>
+        <v/>
+      </c>
+      <c r="C62" s="5">
+        <f>IF(ROUND(B62,4)=1,"OK","CHECK")</f>
+        <v/>
+      </c>
+      <c r="H62" s="33">
+        <f>SUM(H54:H61)</f>
+        <v/>
+      </c>
+      <c r="I62" s="33">
+        <f>SUM(I54:I61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Leads per channel = leases from that channel ÷ its lead-to-lease rate. Shift the lease mix toward channels that convert to cut spend. Leave 2026 actual blank if unknown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Fixed &amp; program costs (property-level)</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="n"/>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="4" t="n"/>
+      <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Monthly ($)</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>One-time / annual ($)</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr"/>
+      <c r="E66" s="16" t="inlineStr"/>
+      <c r="F66" s="16" t="inlineStr"/>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>AI leasing assistant / chat</t>
+        </is>
+      </c>
+      <c r="B67" s="28" t="n">
+        <v>166</v>
+      </c>
+      <c r="C67" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E62" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" s="28" t="n"/>
-      <c r="H62" s="31" t="n">
-        <v>71</v>
-      </c>
-      <c r="I62" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="J62" s="7" t="inlineStr">
-        <is>
-          <t>ACTUAL: sister community, RentCafe, walk-in, unknown, etc. (AptGeo $0 in 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Total (lease mix must = 100%)</t>
-        </is>
-      </c>
-      <c r="B63" s="30">
-        <f>SUM(B54:B62)</f>
-        <v/>
-      </c>
-      <c r="C63" s="5">
-        <f>IF(ROUND(B63,4)=1,"OK","CHECK")</f>
-        <v/>
-      </c>
-      <c r="H63" s="33">
-        <f>SUM(H54:H62)</f>
-        <v/>
-      </c>
-      <c r="I63" s="33">
-        <f>SUM(I54:I62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>Leads per channel = leases from that channel ÷ its lead-to-lease rate. Shift the lease mix toward channels that convert to cut spend. Leave 2026 actual blank if unknown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Fixed &amp; program costs (property-level)</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="4" t="n"/>
-      <c r="E66" s="4" t="n"/>
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="4" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="16" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B67" s="16" t="inlineStr">
-        <is>
-          <t>Monthly ($)</t>
-        </is>
-      </c>
-      <c r="C67" s="16" t="inlineStr">
-        <is>
-          <t>One-time / annual ($)</t>
-        </is>
-      </c>
-      <c r="D67" s="16" t="inlineStr"/>
-      <c r="E67" s="16" t="inlineStr"/>
-      <c r="F67" s="16" t="inlineStr"/>
-      <c r="G67" s="16" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER: e.g. ~$1/unit/mo</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="25" t="inlineStr">
         <is>
-          <t>CRM / lead management (allocated)</t>
+          <t>Reputation management / review software</t>
         </is>
       </c>
       <c r="B68" s="28" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="C68" s="28" t="n">
         <v>0</v>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: e.g. ~$1.50/unit/mo</t>
+          <t>PLACEHOLDER</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>AI leasing assistant / chat</t>
+          <t>Website hosting &amp; maintenance</t>
         </is>
       </c>
       <c r="B69" s="28" t="n">
-        <v>166</v>
+        <v>100</v>
       </c>
       <c r="C69" s="28" t="n">
         <v>0</v>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: e.g. ~$1/unit/mo</t>
+          <t>PLACEHOLDER</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="inlineStr">
         <is>
-          <t>Reputation management / review software</t>
+          <t>Photography / video / virtual tour refresh</t>
         </is>
       </c>
       <c r="B70" s="28" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="C70" s="28" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>PLACEHOLDER: one-time 2027 refresh</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="25" t="inlineStr">
         <is>
-          <t>Website hosting &amp; maintenance</t>
+          <t>Signage &amp; banners</t>
         </is>
       </c>
       <c r="B71" s="28" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C71" s="28" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
@@ -2773,95 +2723,59 @@
     <row r="72">
       <c r="A72" s="25" t="inlineStr">
         <is>
-          <t>Photography / video / virtual tour refresh</t>
+          <t>Print collateral</t>
         </is>
       </c>
       <c r="B72" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C72" s="28" t="n">
-        <v>1500</v>
+        <v>300</v>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER: one-time 2027 refresh</t>
+          <t>PLACEHOLDER</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="25" t="inlineStr">
         <is>
-          <t>Signage &amp; banners</t>
+          <t>Resident events &amp; retention</t>
         </is>
       </c>
       <c r="B73" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C73" s="28" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>PLACEHOLDER: ~4 events/yr; retention is cheaper than replacement</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="25" t="inlineStr">
         <is>
-          <t>Print collateral</t>
+          <t>Freelance / agency support</t>
         </is>
       </c>
       <c r="B74" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C74" s="28" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>Optional: outsourced help for a one-person team</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="25" t="inlineStr">
-        <is>
-          <t>Resident events &amp; retention</t>
-        </is>
-      </c>
-      <c r="B75" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C75" s="28" t="n">
-        <v>3000</v>
-      </c>
       <c r="G75" s="7" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: ~4 events/yr; retention is cheaper than replacement</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="25" t="inlineStr">
-        <is>
-          <t>Freelance / agency support</t>
-        </is>
-      </c>
-      <c r="B76" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C76" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
-        <is>
-          <t>Optional: outsourced help for a one-person team</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="G77" s="7" t="inlineStr">
         <is>
           <t>One-time / annual amounts are spread evenly across 12 months in the Monthly Plan.</t>
         </is>
@@ -2878,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3841,194 +3755,195 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17">
-        <f>Inputs!$A$62</f>
-        <v/>
-      </c>
-      <c r="B21" s="35">
-        <f>IFERROR(B11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="C21" s="35">
-        <f>IFERROR(C11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="D21" s="35">
-        <f>IFERROR(D11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="E21" s="35">
-        <f>IFERROR(E11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="35">
-        <f>IFERROR(F11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="G21" s="35">
-        <f>IFERROR(G11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="H21" s="35">
-        <f>IFERROR(H11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="I21" s="35">
-        <f>IFERROR(I11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="J21" s="35">
-        <f>IFERROR(J11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="K21" s="35">
-        <f>IFERROR(K11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="L21" s="35">
-        <f>IFERROR(L11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="M21" s="35">
-        <f>IFERROR(M11*Inputs!$B$62/Inputs!$C$62,0)</f>
-        <v/>
-      </c>
-      <c r="N21" s="34">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Total leads needed</t>
+        </is>
+      </c>
+      <c r="B21" s="32">
+        <f>SUM(B13:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="32">
+        <f>SUM(C13:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="32">
+        <f>SUM(D13:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="32">
+        <f>SUM(E13:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="32">
+        <f>SUM(F13:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="32">
+        <f>SUM(G13:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="32">
+        <f>SUM(H13:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="32">
+        <f>SUM(I13:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="32">
+        <f>SUM(J13:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="32">
+        <f>SUM(K13:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="32">
+        <f>SUM(L13:L20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="32">
+        <f>SUM(M13:M20)</f>
+        <v/>
+      </c>
+      <c r="N21" s="32">
         <f>SUM(B21:M21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Total leads needed</t>
-        </is>
-      </c>
-      <c r="B22" s="32">
-        <f>SUM(B13:B21)</f>
-        <v/>
-      </c>
-      <c r="C22" s="32">
-        <f>SUM(C13:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="32">
-        <f>SUM(D13:D21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="32">
-        <f>SUM(E13:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="32">
-        <f>SUM(F13:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="32">
-        <f>SUM(G13:G21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="32">
-        <f>SUM(H13:H21)</f>
-        <v/>
-      </c>
-      <c r="I22" s="32">
-        <f>SUM(I13:I21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="32">
-        <f>SUM(J13:J21)</f>
-        <v/>
-      </c>
-      <c r="K22" s="32">
-        <f>SUM(K13:K21)</f>
-        <v/>
-      </c>
-      <c r="L22" s="32">
-        <f>SUM(L13:L21)</f>
-        <v/>
-      </c>
-      <c r="M22" s="32">
-        <f>SUM(M13:M21)</f>
-        <v/>
-      </c>
-      <c r="N22" s="32">
-        <f>SUM(B22:M22)</f>
-        <v/>
-      </c>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Funnel targets</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
+      <c r="M22" s="4" t="n"/>
+      <c r="N22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Funnel targets</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-      <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n"/>
-      <c r="M23" s="4" t="n"/>
-      <c r="N23" s="4" t="n"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Tours needed</t>
+        </is>
+      </c>
+      <c r="B23" s="36">
+        <f>B21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="C23" s="36">
+        <f>C21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="D23" s="36">
+        <f>D21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="E23" s="36">
+        <f>E21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="F23" s="36">
+        <f>F21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="G23" s="36">
+        <f>G21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="H23" s="36">
+        <f>H21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="I23" s="36">
+        <f>I21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="J23" s="36">
+        <f>J21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="K23" s="36">
+        <f>K21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="L23" s="36">
+        <f>L21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="M23" s="36">
+        <f>M21*Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="N23" s="32">
+        <f>SUM(B23:M23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Tours needed</t>
+          <t>Applications needed</t>
         </is>
       </c>
       <c r="B24" s="36">
-        <f>B22*Inputs!$B$21</f>
+        <f>B23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="C24" s="36">
-        <f>C22*Inputs!$B$21</f>
+        <f>C23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="D24" s="36">
-        <f>D22*Inputs!$B$21</f>
+        <f>D23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="E24" s="36">
-        <f>E22*Inputs!$B$21</f>
+        <f>E23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="F24" s="36">
-        <f>F22*Inputs!$B$21</f>
+        <f>F23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="G24" s="36">
-        <f>G22*Inputs!$B$21</f>
+        <f>G23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="H24" s="36">
-        <f>H22*Inputs!$B$21</f>
+        <f>H23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="I24" s="36">
-        <f>I22*Inputs!$B$21</f>
+        <f>I23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="J24" s="36">
-        <f>J22*Inputs!$B$21</f>
+        <f>J23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="K24" s="36">
-        <f>K22*Inputs!$B$21</f>
+        <f>K23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="L24" s="36">
-        <f>L22*Inputs!$B$21</f>
+        <f>L23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="M24" s="36">
-        <f>M22*Inputs!$B$21</f>
+        <f>M23*Inputs!$B$22</f>
         <v/>
       </c>
       <c r="N24" s="32">
@@ -4037,135 +3952,134 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Applications needed</t>
-        </is>
-      </c>
-      <c r="B25" s="36">
-        <f>B24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="C25" s="36">
-        <f>C24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="D25" s="36">
-        <f>D24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="E25" s="36">
-        <f>E24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="F25" s="36">
-        <f>F24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="G25" s="36">
-        <f>G24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="H25" s="36">
-        <f>H24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="I25" s="36">
-        <f>I24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="J25" s="36">
-        <f>J24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="K25" s="36">
-        <f>K24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="L25" s="36">
-        <f>L24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="M25" s="36">
-        <f>M24*Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="N25" s="32">
-        <f>SUM(B25:M25)</f>
-        <v/>
-      </c>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Spend by lead channel ($)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Spend by lead channel ($)</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
+      <c r="A26" s="17">
+        <f>Inputs!$A$54</f>
+        <v/>
+      </c>
+      <c r="B26" s="37">
+        <f>Inputs!$E$54+B13*Inputs!$D$54+B11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="C26" s="37">
+        <f>Inputs!$E$54+C13*Inputs!$D$54+C11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>Inputs!$E$54+D13*Inputs!$D$54+D11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="E26" s="37">
+        <f>Inputs!$E$54+E13*Inputs!$D$54+E11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="F26" s="37">
+        <f>Inputs!$E$54+F13*Inputs!$D$54+F11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="G26" s="37">
+        <f>Inputs!$E$54+G13*Inputs!$D$54+G11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="H26" s="37">
+        <f>Inputs!$E$54+H13*Inputs!$D$54+H11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="I26" s="37">
+        <f>Inputs!$E$54+I13*Inputs!$D$54+I11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="J26" s="37">
+        <f>Inputs!$E$54+J13*Inputs!$D$54+J11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="K26" s="37">
+        <f>Inputs!$E$54+K13*Inputs!$D$54+K11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="L26" s="37">
+        <f>Inputs!$E$54+L13*Inputs!$D$54+L11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="M26" s="37">
+        <f>Inputs!$E$54+M13*Inputs!$D$54+M11*Inputs!$B$54*Inputs!$F$54</f>
+        <v/>
+      </c>
+      <c r="N26" s="38">
+        <f>SUM(B26:M26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="17">
-        <f>Inputs!$A$54</f>
+        <f>Inputs!$A$55</f>
         <v/>
       </c>
       <c r="B27" s="37">
-        <f>Inputs!$E$54+B13*Inputs!$D$54+B11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+B14*Inputs!$D$55+B11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="C27" s="37">
-        <f>Inputs!$E$54+C13*Inputs!$D$54+C11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+C14*Inputs!$D$55+C11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="D27" s="37">
-        <f>Inputs!$E$54+D13*Inputs!$D$54+D11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+D14*Inputs!$D$55+D11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="E27" s="37">
-        <f>Inputs!$E$54+E13*Inputs!$D$54+E11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+E14*Inputs!$D$55+E11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="F27" s="37">
-        <f>Inputs!$E$54+F13*Inputs!$D$54+F11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+F14*Inputs!$D$55+F11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="G27" s="37">
-        <f>Inputs!$E$54+G13*Inputs!$D$54+G11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+G14*Inputs!$D$55+G11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="H27" s="37">
-        <f>Inputs!$E$54+H13*Inputs!$D$54+H11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+H14*Inputs!$D$55+H11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="I27" s="37">
-        <f>Inputs!$E$54+I13*Inputs!$D$54+I11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+I14*Inputs!$D$55+I11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="J27" s="37">
-        <f>Inputs!$E$54+J13*Inputs!$D$54+J11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+J14*Inputs!$D$55+J11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="K27" s="37">
-        <f>Inputs!$E$54+K13*Inputs!$D$54+K11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+K14*Inputs!$D$55+K11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="L27" s="37">
-        <f>Inputs!$E$54+L13*Inputs!$D$54+L11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+L14*Inputs!$D$55+L11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="M27" s="37">
-        <f>Inputs!$E$54+M13*Inputs!$D$54+M11*Inputs!$B$54*Inputs!$F$54</f>
+        <f>Inputs!$E$55+M14*Inputs!$D$55+M11*Inputs!$B$55*Inputs!$F$55</f>
         <v/>
       </c>
       <c r="N27" s="38">
@@ -4175,55 +4089,55 @@
     </row>
     <row r="28">
       <c r="A28" s="17">
-        <f>Inputs!$A$55</f>
+        <f>Inputs!$A$56</f>
         <v/>
       </c>
       <c r="B28" s="37">
-        <f>Inputs!$E$55+B14*Inputs!$D$55+B11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+B15*Inputs!$D$56+B11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="C28" s="37">
-        <f>Inputs!$E$55+C14*Inputs!$D$55+C11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+C15*Inputs!$D$56+C11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="D28" s="37">
-        <f>Inputs!$E$55+D14*Inputs!$D$55+D11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+D15*Inputs!$D$56+D11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="E28" s="37">
-        <f>Inputs!$E$55+E14*Inputs!$D$55+E11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+E15*Inputs!$D$56+E11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="F28" s="37">
-        <f>Inputs!$E$55+F14*Inputs!$D$55+F11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+F15*Inputs!$D$56+F11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="G28" s="37">
-        <f>Inputs!$E$55+G14*Inputs!$D$55+G11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+G15*Inputs!$D$56+G11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="H28" s="37">
-        <f>Inputs!$E$55+H14*Inputs!$D$55+H11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+H15*Inputs!$D$56+H11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="I28" s="37">
-        <f>Inputs!$E$55+I14*Inputs!$D$55+I11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+I15*Inputs!$D$56+I11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="J28" s="37">
-        <f>Inputs!$E$55+J14*Inputs!$D$55+J11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+J15*Inputs!$D$56+J11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="K28" s="37">
-        <f>Inputs!$E$55+K14*Inputs!$D$55+K11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+K15*Inputs!$D$56+K11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="L28" s="37">
-        <f>Inputs!$E$55+L14*Inputs!$D$55+L11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+L15*Inputs!$D$56+L11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="M28" s="37">
-        <f>Inputs!$E$55+M14*Inputs!$D$55+M11*Inputs!$B$55*Inputs!$F$55</f>
+        <f>Inputs!$E$56+M15*Inputs!$D$56+M11*Inputs!$B$56*Inputs!$F$56</f>
         <v/>
       </c>
       <c r="N28" s="38">
@@ -4233,55 +4147,55 @@
     </row>
     <row r="29">
       <c r="A29" s="17">
-        <f>Inputs!$A$56</f>
+        <f>Inputs!$A$57</f>
         <v/>
       </c>
       <c r="B29" s="37">
-        <f>Inputs!$E$56+B15*Inputs!$D$56+B11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+B16*Inputs!$D$57+B11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="C29" s="37">
-        <f>Inputs!$E$56+C15*Inputs!$D$56+C11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+C16*Inputs!$D$57+C11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="D29" s="37">
-        <f>Inputs!$E$56+D15*Inputs!$D$56+D11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+D16*Inputs!$D$57+D11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="E29" s="37">
-        <f>Inputs!$E$56+E15*Inputs!$D$56+E11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+E16*Inputs!$D$57+E11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="F29" s="37">
-        <f>Inputs!$E$56+F15*Inputs!$D$56+F11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+F16*Inputs!$D$57+F11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="G29" s="37">
-        <f>Inputs!$E$56+G15*Inputs!$D$56+G11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+G16*Inputs!$D$57+G11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="H29" s="37">
-        <f>Inputs!$E$56+H15*Inputs!$D$56+H11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+H16*Inputs!$D$57+H11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="I29" s="37">
-        <f>Inputs!$E$56+I15*Inputs!$D$56+I11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+I16*Inputs!$D$57+I11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="J29" s="37">
-        <f>Inputs!$E$56+J15*Inputs!$D$56+J11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+J16*Inputs!$D$57+J11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="K29" s="37">
-        <f>Inputs!$E$56+K15*Inputs!$D$56+K11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+K16*Inputs!$D$57+K11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="L29" s="37">
-        <f>Inputs!$E$56+L15*Inputs!$D$56+L11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+L16*Inputs!$D$57+L11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="M29" s="37">
-        <f>Inputs!$E$56+M15*Inputs!$D$56+M11*Inputs!$B$56*Inputs!$F$56</f>
+        <f>Inputs!$E$57+M16*Inputs!$D$57+M11*Inputs!$B$57*Inputs!$F$57</f>
         <v/>
       </c>
       <c r="N29" s="38">
@@ -4291,55 +4205,55 @@
     </row>
     <row r="30">
       <c r="A30" s="17">
-        <f>Inputs!$A$57</f>
+        <f>Inputs!$A$58</f>
         <v/>
       </c>
       <c r="B30" s="37">
-        <f>Inputs!$E$57+B16*Inputs!$D$57+B11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+B17*Inputs!$D$58+B11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="C30" s="37">
-        <f>Inputs!$E$57+C16*Inputs!$D$57+C11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+C17*Inputs!$D$58+C11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="D30" s="37">
-        <f>Inputs!$E$57+D16*Inputs!$D$57+D11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+D17*Inputs!$D$58+D11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="E30" s="37">
-        <f>Inputs!$E$57+E16*Inputs!$D$57+E11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+E17*Inputs!$D$58+E11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="F30" s="37">
-        <f>Inputs!$E$57+F16*Inputs!$D$57+F11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+F17*Inputs!$D$58+F11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="G30" s="37">
-        <f>Inputs!$E$57+G16*Inputs!$D$57+G11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+G17*Inputs!$D$58+G11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="H30" s="37">
-        <f>Inputs!$E$57+H16*Inputs!$D$57+H11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+H17*Inputs!$D$58+H11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="I30" s="37">
-        <f>Inputs!$E$57+I16*Inputs!$D$57+I11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+I17*Inputs!$D$58+I11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="J30" s="37">
-        <f>Inputs!$E$57+J16*Inputs!$D$57+J11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+J17*Inputs!$D$58+J11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="K30" s="37">
-        <f>Inputs!$E$57+K16*Inputs!$D$57+K11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+K17*Inputs!$D$58+K11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="L30" s="37">
-        <f>Inputs!$E$57+L16*Inputs!$D$57+L11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+L17*Inputs!$D$58+L11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="M30" s="37">
-        <f>Inputs!$E$57+M16*Inputs!$D$57+M11*Inputs!$B$57*Inputs!$F$57</f>
+        <f>Inputs!$E$58+M17*Inputs!$D$58+M11*Inputs!$B$58*Inputs!$F$58</f>
         <v/>
       </c>
       <c r="N30" s="38">
@@ -4349,55 +4263,55 @@
     </row>
     <row r="31">
       <c r="A31" s="17">
-        <f>Inputs!$A$58</f>
+        <f>Inputs!$A$59</f>
         <v/>
       </c>
       <c r="B31" s="37">
-        <f>Inputs!$E$58+B17*Inputs!$D$58+B11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+B18*Inputs!$D$59+B11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="C31" s="37">
-        <f>Inputs!$E$58+C17*Inputs!$D$58+C11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+C18*Inputs!$D$59+C11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="D31" s="37">
-        <f>Inputs!$E$58+D17*Inputs!$D$58+D11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+D18*Inputs!$D$59+D11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="E31" s="37">
-        <f>Inputs!$E$58+E17*Inputs!$D$58+E11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+E18*Inputs!$D$59+E11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="F31" s="37">
-        <f>Inputs!$E$58+F17*Inputs!$D$58+F11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+F18*Inputs!$D$59+F11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="G31" s="37">
-        <f>Inputs!$E$58+G17*Inputs!$D$58+G11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+G18*Inputs!$D$59+G11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="H31" s="37">
-        <f>Inputs!$E$58+H17*Inputs!$D$58+H11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+H18*Inputs!$D$59+H11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="I31" s="37">
-        <f>Inputs!$E$58+I17*Inputs!$D$58+I11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+I18*Inputs!$D$59+I11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="J31" s="37">
-        <f>Inputs!$E$58+J17*Inputs!$D$58+J11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+J18*Inputs!$D$59+J11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="K31" s="37">
-        <f>Inputs!$E$58+K17*Inputs!$D$58+K11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+K18*Inputs!$D$59+K11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="L31" s="37">
-        <f>Inputs!$E$58+L17*Inputs!$D$58+L11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+L18*Inputs!$D$59+L11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="M31" s="37">
-        <f>Inputs!$E$58+M17*Inputs!$D$58+M11*Inputs!$B$58*Inputs!$F$58</f>
+        <f>Inputs!$E$59+M18*Inputs!$D$59+M11*Inputs!$B$59*Inputs!$F$59</f>
         <v/>
       </c>
       <c r="N31" s="38">
@@ -4407,55 +4321,55 @@
     </row>
     <row r="32">
       <c r="A32" s="17">
-        <f>Inputs!$A$59</f>
+        <f>Inputs!$A$60</f>
         <v/>
       </c>
       <c r="B32" s="37">
-        <f>Inputs!$E$59+B18*Inputs!$D$59+B11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+B19*Inputs!$D$60+B11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="C32" s="37">
-        <f>Inputs!$E$59+C18*Inputs!$D$59+C11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+C19*Inputs!$D$60+C11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="D32" s="37">
-        <f>Inputs!$E$59+D18*Inputs!$D$59+D11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+D19*Inputs!$D$60+D11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="E32" s="37">
-        <f>Inputs!$E$59+E18*Inputs!$D$59+E11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+E19*Inputs!$D$60+E11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="F32" s="37">
-        <f>Inputs!$E$59+F18*Inputs!$D$59+F11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+F19*Inputs!$D$60+F11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="G32" s="37">
-        <f>Inputs!$E$59+G18*Inputs!$D$59+G11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+G19*Inputs!$D$60+G11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="H32" s="37">
-        <f>Inputs!$E$59+H18*Inputs!$D$59+H11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+H19*Inputs!$D$60+H11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="I32" s="37">
-        <f>Inputs!$E$59+I18*Inputs!$D$59+I11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+I19*Inputs!$D$60+I11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="J32" s="37">
-        <f>Inputs!$E$59+J18*Inputs!$D$59+J11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+J19*Inputs!$D$60+J11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="K32" s="37">
-        <f>Inputs!$E$59+K18*Inputs!$D$59+K11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+K19*Inputs!$D$60+K11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="L32" s="37">
-        <f>Inputs!$E$59+L18*Inputs!$D$59+L11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+L19*Inputs!$D$60+L11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="M32" s="37">
-        <f>Inputs!$E$59+M18*Inputs!$D$59+M11*Inputs!$B$59*Inputs!$F$59</f>
+        <f>Inputs!$E$60+M19*Inputs!$D$60+M11*Inputs!$B$60*Inputs!$F$60</f>
         <v/>
       </c>
       <c r="N32" s="38">
@@ -4465,55 +4379,55 @@
     </row>
     <row r="33">
       <c r="A33" s="17">
-        <f>Inputs!$A$60</f>
+        <f>Inputs!$A$61</f>
         <v/>
       </c>
       <c r="B33" s="37">
-        <f>Inputs!$E$60+B19*Inputs!$D$60+B11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+B20*Inputs!$D$61+B11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="C33" s="37">
-        <f>Inputs!$E$60+C19*Inputs!$D$60+C11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+C20*Inputs!$D$61+C11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="D33" s="37">
-        <f>Inputs!$E$60+D19*Inputs!$D$60+D11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+D20*Inputs!$D$61+D11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="E33" s="37">
-        <f>Inputs!$E$60+E19*Inputs!$D$60+E11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+E20*Inputs!$D$61+E11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="F33" s="37">
-        <f>Inputs!$E$60+F19*Inputs!$D$60+F11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+F20*Inputs!$D$61+F11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="G33" s="37">
-        <f>Inputs!$E$60+G19*Inputs!$D$60+G11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+G20*Inputs!$D$61+G11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="H33" s="37">
-        <f>Inputs!$E$60+H19*Inputs!$D$60+H11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+H20*Inputs!$D$61+H11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="I33" s="37">
-        <f>Inputs!$E$60+I19*Inputs!$D$60+I11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+I20*Inputs!$D$61+I11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="J33" s="37">
-        <f>Inputs!$E$60+J19*Inputs!$D$60+J11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+J20*Inputs!$D$61+J11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="K33" s="37">
-        <f>Inputs!$E$60+K19*Inputs!$D$60+K11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+K20*Inputs!$D$61+K11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="L33" s="37">
-        <f>Inputs!$E$60+L19*Inputs!$D$60+L11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+L20*Inputs!$D$61+L11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="M33" s="37">
-        <f>Inputs!$E$60+M19*Inputs!$D$60+M11*Inputs!$B$60*Inputs!$F$60</f>
+        <f>Inputs!$E$61+M20*Inputs!$D$61+M11*Inputs!$B$61*Inputs!$F$61</f>
         <v/>
       </c>
       <c r="N33" s="38">
@@ -4522,56 +4436,57 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="17">
-        <f>Inputs!$A$61</f>
-        <v/>
-      </c>
-      <c r="B34" s="37">
-        <f>Inputs!$E$61+B20*Inputs!$D$61+B11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="C34" s="37">
-        <f>Inputs!$E$61+C20*Inputs!$D$61+C11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="D34" s="37">
-        <f>Inputs!$E$61+D20*Inputs!$D$61+D11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="E34" s="37">
-        <f>Inputs!$E$61+E20*Inputs!$D$61+E11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="F34" s="37">
-        <f>Inputs!$E$61+F20*Inputs!$D$61+F11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="G34" s="37">
-        <f>Inputs!$E$61+G20*Inputs!$D$61+G11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="H34" s="37">
-        <f>Inputs!$E$61+H20*Inputs!$D$61+H11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="I34" s="37">
-        <f>Inputs!$E$61+I20*Inputs!$D$61+I11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="J34" s="37">
-        <f>Inputs!$E$61+J20*Inputs!$D$61+J11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="K34" s="37">
-        <f>Inputs!$E$61+K20*Inputs!$D$61+K11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="L34" s="37">
-        <f>Inputs!$E$61+L20*Inputs!$D$61+L11*Inputs!$B$61*Inputs!$F$61</f>
-        <v/>
-      </c>
-      <c r="M34" s="37">
-        <f>Inputs!$E$61+M20*Inputs!$D$61+M11*Inputs!$B$61*Inputs!$F$61</f>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Channel subtotal</t>
+        </is>
+      </c>
+      <c r="B34" s="38">
+        <f>SUM(B26:B33)</f>
+        <v/>
+      </c>
+      <c r="C34" s="38">
+        <f>SUM(C26:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="38">
+        <f>SUM(D26:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="38">
+        <f>SUM(E26:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="38">
+        <f>SUM(F26:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="38">
+        <f>SUM(G26:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="38">
+        <f>SUM(H26:H33)</f>
+        <v/>
+      </c>
+      <c r="I34" s="38">
+        <f>SUM(I26:I33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="38">
+        <f>SUM(J26:J33)</f>
+        <v/>
+      </c>
+      <c r="K34" s="38">
+        <f>SUM(K26:K33)</f>
+        <v/>
+      </c>
+      <c r="L34" s="38">
+        <f>SUM(L26:L33)</f>
+        <v/>
+      </c>
+      <c r="M34" s="38">
+        <f>SUM(M26:M33)</f>
         <v/>
       </c>
       <c r="N34" s="38">
@@ -4580,115 +4495,76 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17">
-        <f>Inputs!$A$62</f>
-        <v/>
-      </c>
-      <c r="B35" s="37">
-        <f>Inputs!$E$62+B21*Inputs!$D$62+B11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="C35" s="37">
-        <f>Inputs!$E$62+C21*Inputs!$D$62+C11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="D35" s="37">
-        <f>Inputs!$E$62+D21*Inputs!$D$62+D11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="E35" s="37">
-        <f>Inputs!$E$62+E21*Inputs!$D$62+E11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="F35" s="37">
-        <f>Inputs!$E$62+F21*Inputs!$D$62+F11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="G35" s="37">
-        <f>Inputs!$E$62+G21*Inputs!$D$62+G11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="H35" s="37">
-        <f>Inputs!$E$62+H21*Inputs!$D$62+H11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="I35" s="37">
-        <f>Inputs!$E$62+I21*Inputs!$D$62+I11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="J35" s="37">
-        <f>Inputs!$E$62+J21*Inputs!$D$62+J11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="K35" s="37">
-        <f>Inputs!$E$62+K21*Inputs!$D$62+K11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="L35" s="37">
-        <f>Inputs!$E$62+L21*Inputs!$D$62+L11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="M35" s="37">
-        <f>Inputs!$E$62+M21*Inputs!$D$62+M11*Inputs!$B$62*Inputs!$F$62</f>
-        <v/>
-      </c>
-      <c r="N35" s="38">
-        <f>SUM(B35:M35)</f>
-        <v/>
-      </c>
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Fixed, program &amp; retention costs ($)</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Channel subtotal</t>
-        </is>
-      </c>
-      <c r="B36" s="38">
-        <f>SUM(B27:B35)</f>
-        <v/>
-      </c>
-      <c r="C36" s="38">
-        <f>SUM(C27:C35)</f>
-        <v/>
-      </c>
-      <c r="D36" s="38">
-        <f>SUM(D27:D35)</f>
-        <v/>
-      </c>
-      <c r="E36" s="38">
-        <f>SUM(E27:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="38">
-        <f>SUM(F27:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="38">
-        <f>SUM(G27:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="38">
-        <f>SUM(H27:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="38">
-        <f>SUM(I27:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="38">
-        <f>SUM(J27:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="38">
-        <f>SUM(K27:K35)</f>
-        <v/>
-      </c>
-      <c r="L36" s="38">
-        <f>SUM(L27:L35)</f>
-        <v/>
-      </c>
-      <c r="M36" s="38">
-        <f>SUM(M27:M35)</f>
+      <c r="A36" s="17">
+        <f>Inputs!$A$67</f>
+        <v/>
+      </c>
+      <c r="B36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="C36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="D36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="E36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="F36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="G36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="H36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="I36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="J36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="K36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="L36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
+        <v/>
+      </c>
+      <c r="M36" s="37">
+        <f>Inputs!$B$67+Inputs!$C$67/12</f>
         <v/>
       </c>
       <c r="N36" s="38">
@@ -4697,76 +4573,114 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Fixed, program &amp; retention costs ($)</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="n"/>
-      <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4" t="n"/>
+      <c r="A37" s="17">
+        <f>Inputs!$A$68</f>
+        <v/>
+      </c>
+      <c r="B37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="C37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="D37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="E37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="F37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="G37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="H37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="I37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="J37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="K37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="L37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="M37" s="37">
+        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <v/>
+      </c>
+      <c r="N37" s="38">
+        <f>SUM(B37:M37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17">
-        <f>Inputs!$A$68</f>
+        <f>Inputs!$A$69</f>
         <v/>
       </c>
       <c r="B38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="C38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="D38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="E38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="F38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="G38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="H38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="I38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="J38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="K38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="L38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="M38" s="37">
-        <f>Inputs!$B$68+Inputs!$C$68/12</f>
+        <f>Inputs!$B$69+Inputs!$C$69/12</f>
         <v/>
       </c>
       <c r="N38" s="38">
@@ -4776,55 +4690,55 @@
     </row>
     <row r="39">
       <c r="A39" s="17">
-        <f>Inputs!$A$69</f>
+        <f>Inputs!$A$70</f>
         <v/>
       </c>
       <c r="B39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="C39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="D39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="E39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="F39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="G39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="H39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="I39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="J39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="K39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="L39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="M39" s="37">
-        <f>Inputs!$B$69+Inputs!$C$69/12</f>
+        <f>Inputs!$B$70+Inputs!$C$70/12</f>
         <v/>
       </c>
       <c r="N39" s="38">
@@ -4834,55 +4748,55 @@
     </row>
     <row r="40">
       <c r="A40" s="17">
-        <f>Inputs!$A$70</f>
+        <f>Inputs!$A$71</f>
         <v/>
       </c>
       <c r="B40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="C40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="D40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="E40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="F40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="G40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="H40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="I40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="J40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="K40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="L40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="M40" s="37">
-        <f>Inputs!$B$70+Inputs!$C$70/12</f>
+        <f>Inputs!$B$71+Inputs!$C$71/12</f>
         <v/>
       </c>
       <c r="N40" s="38">
@@ -4892,55 +4806,55 @@
     </row>
     <row r="41">
       <c r="A41" s="17">
-        <f>Inputs!$A$71</f>
+        <f>Inputs!$A$72</f>
         <v/>
       </c>
       <c r="B41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="C41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="D41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="E41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="F41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="G41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="H41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="I41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="J41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="K41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="L41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="M41" s="37">
-        <f>Inputs!$B$71+Inputs!$C$71/12</f>
+        <f>Inputs!$B$72+Inputs!$C$72/12</f>
         <v/>
       </c>
       <c r="N41" s="38">
@@ -4950,55 +4864,55 @@
     </row>
     <row r="42">
       <c r="A42" s="17">
-        <f>Inputs!$A$72</f>
+        <f>Inputs!$A$73</f>
         <v/>
       </c>
       <c r="B42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="C42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="D42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="E42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="F42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="G42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="H42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="I42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="J42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="K42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="L42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="M42" s="37">
-        <f>Inputs!$B$72+Inputs!$C$72/12</f>
+        <f>Inputs!$B$73+Inputs!$C$73/12</f>
         <v/>
       </c>
       <c r="N42" s="38">
@@ -5008,55 +4922,55 @@
     </row>
     <row r="43">
       <c r="A43" s="17">
-        <f>Inputs!$A$73</f>
+        <f>Inputs!$A$74</f>
         <v/>
       </c>
       <c r="B43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="C43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="D43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="E43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="F43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="G43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="H43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="I43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="J43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="K43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="L43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="M43" s="37">
-        <f>Inputs!$B$73+Inputs!$C$73/12</f>
+        <f>Inputs!$B$74+Inputs!$C$74/12</f>
         <v/>
       </c>
       <c r="N43" s="38">
@@ -5065,56 +4979,57 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17">
-        <f>Inputs!$A$74</f>
-        <v/>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Renewal incentives</t>
+        </is>
       </c>
       <c r="B44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>B7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="C44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>C7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="D44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>D7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="E44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>E7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="F44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>F7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="G44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>G7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="H44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>H7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="I44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>I7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="J44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>J7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="K44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>K7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="L44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>L7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="M44" s="37">
-        <f>Inputs!$B$74+Inputs!$C$74/12</f>
+        <f>M7*Inputs!$B$18</f>
         <v/>
       </c>
       <c r="N44" s="38">
@@ -5123,56 +5038,57 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="17">
-        <f>Inputs!$A$75</f>
-        <v/>
-      </c>
-      <c r="B45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="C45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="D45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="E45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="F45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="G45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="H45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="I45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="J45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="K45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="L45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
-        <v/>
-      </c>
-      <c r="M45" s="37">
-        <f>Inputs!$B$75+Inputs!$C$75/12</f>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Fixed &amp; retention subtotal</t>
+        </is>
+      </c>
+      <c r="B45" s="38">
+        <f>SUM(B36:B44)</f>
+        <v/>
+      </c>
+      <c r="C45" s="38">
+        <f>SUM(C36:C44)</f>
+        <v/>
+      </c>
+      <c r="D45" s="38">
+        <f>SUM(D36:D44)</f>
+        <v/>
+      </c>
+      <c r="E45" s="38">
+        <f>SUM(E36:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="38">
+        <f>SUM(F36:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="38">
+        <f>SUM(G36:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="38">
+        <f>SUM(H36:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="38">
+        <f>SUM(I36:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="38">
+        <f>SUM(J36:J44)</f>
+        <v/>
+      </c>
+      <c r="K45" s="38">
+        <f>SUM(K36:K44)</f>
+        <v/>
+      </c>
+      <c r="L45" s="38">
+        <f>SUM(L36:L44)</f>
+        <v/>
+      </c>
+      <c r="M45" s="38">
+        <f>SUM(M36:M44)</f>
         <v/>
       </c>
       <c r="N45" s="38">
@@ -5181,115 +5097,77 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="17">
-        <f>Inputs!$A$76</f>
-        <v/>
-      </c>
-      <c r="B46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="C46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="D46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="E46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="F46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="G46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="H46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="I46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="J46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="K46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="L46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="M46" s="37">
-        <f>Inputs!$B$76+Inputs!$C$76/12</f>
-        <v/>
-      </c>
-      <c r="N46" s="38">
-        <f>SUM(B46:M46)</f>
-        <v/>
-      </c>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+      <c r="J46" s="4" t="n"/>
+      <c r="K46" s="4" t="n"/>
+      <c r="L46" s="4" t="n"/>
+      <c r="M46" s="4" t="n"/>
+      <c r="N46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Renewal incentives</t>
+          <t>Budget before contingency</t>
         </is>
       </c>
       <c r="B47" s="37">
-        <f>B7*Inputs!$B$18</f>
+        <f>B34+B45</f>
         <v/>
       </c>
       <c r="C47" s="37">
-        <f>C7*Inputs!$B$18</f>
+        <f>C34+C45</f>
         <v/>
       </c>
       <c r="D47" s="37">
-        <f>D7*Inputs!$B$18</f>
+        <f>D34+D45</f>
         <v/>
       </c>
       <c r="E47" s="37">
-        <f>E7*Inputs!$B$18</f>
+        <f>E34+E45</f>
         <v/>
       </c>
       <c r="F47" s="37">
-        <f>F7*Inputs!$B$18</f>
+        <f>F34+F45</f>
         <v/>
       </c>
       <c r="G47" s="37">
-        <f>G7*Inputs!$B$18</f>
+        <f>G34+G45</f>
         <v/>
       </c>
       <c r="H47" s="37">
-        <f>H7*Inputs!$B$18</f>
+        <f>H34+H45</f>
         <v/>
       </c>
       <c r="I47" s="37">
-        <f>I7*Inputs!$B$18</f>
+        <f>I34+I45</f>
         <v/>
       </c>
       <c r="J47" s="37">
-        <f>J7*Inputs!$B$18</f>
+        <f>J34+J45</f>
         <v/>
       </c>
       <c r="K47" s="37">
-        <f>K7*Inputs!$B$18</f>
+        <f>K34+K45</f>
         <v/>
       </c>
       <c r="L47" s="37">
-        <f>L7*Inputs!$B$18</f>
+        <f>L34+L45</f>
         <v/>
       </c>
       <c r="M47" s="37">
-        <f>M7*Inputs!$B$18</f>
+        <f>M34+M45</f>
         <v/>
       </c>
       <c r="N47" s="38">
@@ -5298,57 +5176,57 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Fixed &amp; retention subtotal</t>
-        </is>
-      </c>
-      <c r="B48" s="38">
-        <f>SUM(B38:B47)</f>
-        <v/>
-      </c>
-      <c r="C48" s="38">
-        <f>SUM(C38:C47)</f>
-        <v/>
-      </c>
-      <c r="D48" s="38">
-        <f>SUM(D38:D47)</f>
-        <v/>
-      </c>
-      <c r="E48" s="38">
-        <f>SUM(E38:E47)</f>
-        <v/>
-      </c>
-      <c r="F48" s="38">
-        <f>SUM(F38:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="38">
-        <f>SUM(G38:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="38">
-        <f>SUM(H38:H47)</f>
-        <v/>
-      </c>
-      <c r="I48" s="38">
-        <f>SUM(I38:I47)</f>
-        <v/>
-      </c>
-      <c r="J48" s="38">
-        <f>SUM(J38:J47)</f>
-        <v/>
-      </c>
-      <c r="K48" s="38">
-        <f>SUM(K38:K47)</f>
-        <v/>
-      </c>
-      <c r="L48" s="38">
-        <f>SUM(L38:L47)</f>
-        <v/>
-      </c>
-      <c r="M48" s="38">
-        <f>SUM(M38:M47)</f>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B48" s="37">
+        <f>B47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="C48" s="37">
+        <f>C47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="D48" s="37">
+        <f>D47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="E48" s="37">
+        <f>E47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="F48" s="37">
+        <f>F47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="G48" s="37">
+        <f>G47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="H48" s="37">
+        <f>H47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="I48" s="37">
+        <f>I47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="J48" s="37">
+        <f>J47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="K48" s="37">
+        <f>K47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="L48" s="37">
+        <f>L47*Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="M48" s="37">
+        <f>M47*Inputs!$B$33</f>
         <v/>
       </c>
       <c r="N48" s="38">
@@ -5357,199 +5235,61 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
-      <c r="J49" s="4" t="n"/>
-      <c r="K49" s="4" t="n"/>
-      <c r="L49" s="4" t="n"/>
-      <c r="M49" s="4" t="n"/>
-      <c r="N49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>Budget before contingency</t>
-        </is>
-      </c>
-      <c r="B50" s="37">
-        <f>B36+B48</f>
-        <v/>
-      </c>
-      <c r="C50" s="37">
-        <f>C36+C48</f>
-        <v/>
-      </c>
-      <c r="D50" s="37">
-        <f>D36+D48</f>
-        <v/>
-      </c>
-      <c r="E50" s="37">
-        <f>E36+E48</f>
-        <v/>
-      </c>
-      <c r="F50" s="37">
-        <f>F36+F48</f>
-        <v/>
-      </c>
-      <c r="G50" s="37">
-        <f>G36+G48</f>
-        <v/>
-      </c>
-      <c r="H50" s="37">
-        <f>H36+H48</f>
-        <v/>
-      </c>
-      <c r="I50" s="37">
-        <f>I36+I48</f>
-        <v/>
-      </c>
-      <c r="J50" s="37">
-        <f>J36+J48</f>
-        <v/>
-      </c>
-      <c r="K50" s="37">
-        <f>K36+K48</f>
-        <v/>
-      </c>
-      <c r="L50" s="37">
-        <f>L36+L48</f>
-        <v/>
-      </c>
-      <c r="M50" s="37">
-        <f>M36+M48</f>
-        <v/>
-      </c>
-      <c r="N50" s="38">
-        <f>SUM(B50:M50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B51" s="37">
-        <f>B50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="C51" s="37">
-        <f>C50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="D51" s="37">
-        <f>D50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="E51" s="37">
-        <f>E50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="F51" s="37">
-        <f>F50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="G51" s="37">
-        <f>G50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="H51" s="37">
-        <f>H50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="I51" s="37">
-        <f>I50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="J51" s="37">
-        <f>J50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="K51" s="37">
-        <f>K50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="L51" s="37">
-        <f>L50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="M51" s="37">
-        <f>M50*Inputs!$B$33</f>
-        <v/>
-      </c>
-      <c r="N51" s="38">
-        <f>SUM(B51:M51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="21" t="inlineStr">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>TOTAL MARKETING BUDGET</t>
         </is>
       </c>
-      <c r="B52" s="22">
-        <f>B50+B51</f>
-        <v/>
-      </c>
-      <c r="C52" s="22">
-        <f>C50+C51</f>
-        <v/>
-      </c>
-      <c r="D52" s="22">
-        <f>D50+D51</f>
-        <v/>
-      </c>
-      <c r="E52" s="22">
-        <f>E50+E51</f>
-        <v/>
-      </c>
-      <c r="F52" s="22">
-        <f>F50+F51</f>
-        <v/>
-      </c>
-      <c r="G52" s="22">
-        <f>G50+G51</f>
-        <v/>
-      </c>
-      <c r="H52" s="22">
-        <f>H50+H51</f>
-        <v/>
-      </c>
-      <c r="I52" s="22">
-        <f>I50+I51</f>
-        <v/>
-      </c>
-      <c r="J52" s="22">
-        <f>J50+J51</f>
-        <v/>
-      </c>
-      <c r="K52" s="22">
-        <f>K50+K51</f>
-        <v/>
-      </c>
-      <c r="L52" s="22">
-        <f>L50+L51</f>
-        <v/>
-      </c>
-      <c r="M52" s="22">
-        <f>M50+M51</f>
-        <v/>
-      </c>
-      <c r="N52" s="22">
-        <f>SUM(B52:M52)</f>
+      <c r="B49" s="22">
+        <f>B47+B48</f>
+        <v/>
+      </c>
+      <c r="C49" s="22">
+        <f>C47+C48</f>
+        <v/>
+      </c>
+      <c r="D49" s="22">
+        <f>D47+D48</f>
+        <v/>
+      </c>
+      <c r="E49" s="22">
+        <f>E47+E48</f>
+        <v/>
+      </c>
+      <c r="F49" s="22">
+        <f>F47+F48</f>
+        <v/>
+      </c>
+      <c r="G49" s="22">
+        <f>G47+G48</f>
+        <v/>
+      </c>
+      <c r="H49" s="22">
+        <f>H47+H48</f>
+        <v/>
+      </c>
+      <c r="I49" s="22">
+        <f>I47+I48</f>
+        <v/>
+      </c>
+      <c r="J49" s="22">
+        <f>J47+J48</f>
+        <v/>
+      </c>
+      <c r="K49" s="22">
+        <f>K47+K48</f>
+        <v/>
+      </c>
+      <c r="L49" s="22">
+        <f>L47+L48</f>
+        <v/>
+      </c>
+      <c r="M49" s="22">
+        <f>M47+M48</f>
+        <v/>
+      </c>
+      <c r="N49" s="22">
+        <f>SUM(B49:M49)</f>
         <v/>
       </c>
     </row>
@@ -5662,35 +5402,35 @@
     <row r="16">
       <c r="A16" s="40" t="inlineStr">
         <is>
-          <t>Done from the WAR: rent, occupancy, renewal rate, lease breaks, funnel, lead sources, days vacant.</t>
+          <t>Excluded per user: Rently and CRM costs. Apartment List folded into All other.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="40" t="inlineStr">
         <is>
-          <t>Done from the 2026 Ad Spend Tracking sheet: Digible, Zillow, CoStar (cancelled 9/30/26), AptGeo and website spend.</t>
+          <t>Done from the WAR: rent, occupancy, renewal rate, lease breaks, funnel, lead sources, days vacant.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="40" t="inlineStr">
         <is>
-          <t>1. 2027 price changes from Digible and Zillow; whether Rently, MLS or Apartment List are billed somewhere else.</t>
+          <t>Done from the 2026 Ad Spend Tracking sheet: Digible, Zillow, CoStar (cancelled 9/30/26), AptGeo and website spend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="40" t="inlineStr">
         <is>
-          <t>2. Digible's lead and lease attribution report (WAR may credit their ads to Property Website).</t>
+          <t>1. Digible's lead and lease attribution report (WAR may credit their ads to Property Website).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="40" t="inlineStr">
         <is>
-          <t>3. Fixed-cost items: CRM, AI leasing, reputation, website, photography, signage, events.</t>
+          <t>2. Fixed-cost items: AI leasing, reputation, website, photography, signage, events.</t>
         </is>
       </c>
     </row>

</xml_diff>